<commit_message>
hoàn thiện và kiểm thử file đặc tả
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThongTin" sheetId="1" r:id="R773cf52d4da04685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YeuCauChucNang" sheetId="2" r:id="R9092c14441c840cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YeuCauPhiChucNang" sheetId="3" r:id="R2eb4de489f6649d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RangBuoc" sheetId="4" r:id="R7e9b826e8af74dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoHinhTrangThai" sheetId="5" r:id="R3250bc9ebd794f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThuocTinhAnToan" sheetId="6" r:id="Ra58f32f8493b4d12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoaiTruLanNhau" sheetId="7" r:id="R5cef1ec9caf14151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HamSinhMa" sheetId="8" r:id="R2bf1d3e36f1c4b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KiemTraSoHoc" sheetId="9" r:id="R6c39ad41364046e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCase" sheetId="10" r:id="Rffca24bf5cf34bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThongTin" sheetId="1" r:id="Rab9a2bb1509b4c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YeuCauChucNang" sheetId="2" r:id="R736703aaa85d4afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YeuCauPhiChucNang" sheetId="3" r:id="R0af1a5f42bd34e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RangBuoc" sheetId="4" r:id="Ree38e5f108114394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MoHinhTrangThai" sheetId="5" r:id="R47dd4da5a5874694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThuocTinhAnToan" sheetId="6" r:id="R13e1ad3616b24377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoaiTruLanNhau" sheetId="7" r:id="Ra984c7c65aca4b58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HamSinhMa" sheetId="8" r:id="R6fd055f6cda246f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KiemTraSoHoc" sheetId="9" r:id="R9d915c8e81aa427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCase" sheetId="10" r:id="R8f4eeb1519bd4f8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -37,6 +37,11 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -87,7 +92,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -116,6 +121,16 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -353,19 +368,19 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>name</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>order_payment_microservice_security</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>Đặc tả kiểm chứng hình thức cho luồng Order-Payment: state machine có xử lý sự cố và phục hồi, safety/liveness, idempotency, serialization payment-cancel, bounded retry, compensation refund, SMT số học và mô hình C về an toàn bộ nhớ.</x:v>
+      <x:c r="B3" s="11" t="str">
+        <x:v>Đặc tả Order-Payment tương thích Spec Verification Lab: kiểm soát truy cập, hai state machine Order/Payment, tồn kho, idempotency, UNKNOWN/reconciliation, bounded retry, refund compensation, concurrency, SMT số học, fuzzing và mô hình C về an toàn bộ nhớ.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -410,500 +425,672 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>TC-1</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>REQ-1</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>Từ chối truy cập API được bảo vệ khi không có JWT</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="11" t="str">
         <x:v>Ứng dụng chạy, request không có Authorization header</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="str">
+      <x:c r="E2" s="11" t="str">
         <x:v>Gọi GET /api/orders/mine
 Gọi GET /api/cart/user/1</x:v>
       </x:c>
-      <x:c r="F2" s="5" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>HTTP 401 cho cả hai request; không trả dữ liệu nghiệp vụ</x:v>
       </x:c>
-      <x:c r="G2" s="5" t="str">
+      <x:c r="G2" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>TC-2</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>REQ-2</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
         <x:v>Chặn truy cập chéo người dùng</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="D3" s="11" t="str">
         <x:v>Có JWT user A và Order/Cart thuộc user B</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="str">
+      <x:c r="E3" s="11" t="str">
         <x:v>Dùng JWT A đọc order B
 Dùng JWT A sửa hoặc xóa cart item của B</x:v>
       </x:c>
-      <x:c r="F3" s="5" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>HTTP 403; Order/Cart của B không thay đổi</x:v>
       </x:c>
-      <x:c r="G3" s="5" t="str">
+      <x:c r="G3" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>TC-3</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>REQ-3, REQ-4</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="C4" s="11" t="str">
         <x:v>Không chấp nhận giá do client sửa</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str">
+      <x:c r="D4" s="11" t="str">
         <x:v>Product giá 25, stock 10</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="str">
+      <x:c r="E4" s="11" t="str">
         <x:v>Tạo Order quantity=2, UnitPrice=1, TotalAmount=2</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>ArgumentException/HTTP 400; không tạo Order và stock vẫn là 10</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="str">
+      <x:c r="G4" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>TC-4</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>REQ-3, REQ-5</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>Tạo đơn hợp lệ bằng giá server</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>Product giá 25, stock 10</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Tạo Order quantity=2, UnitPrice=25, TotalAmount=50</x:v>
       </x:c>
-      <x:c r="F5" s="5" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>Order ở PAYMENT_PENDING, TotalAmount=50, UnitPrice=25, stock còn 8</x:v>
       </x:c>
-      <x:c r="G5" s="5" t="str">
+      <x:c r="G5" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>TC-5</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>REQ-5, REQ-6</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>Không thanh toán Order đã CANCELLED</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>Order CANCELLED, TotalAmount=100</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="str">
+      <x:c r="E6" s="11" t="str">
         <x:v>Tạo Payment Amount=100 với idempotency key mới</x:v>
       </x:c>
-      <x:c r="F6" s="5" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>Bị từ chối; không có Payment và Order vẫn CANCELLED</x:v>
       </x:c>
-      <x:c r="G6" s="5" t="str">
+      <x:c r="G6" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>TC-6</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>REQ-6</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
         <x:v>Payment phải bằng đúng tổng Order</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="11" t="str">
         <x:v>Order PAYMENT_PENDING, TotalAmount=100</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="str">
+      <x:c r="E7" s="11" t="str">
         <x:v>Tạo Payment Amount=99</x:v>
       </x:c>
-      <x:c r="F7" s="5" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>Bị từ chối; Order vẫn PAYMENT_PENDING</x:v>
       </x:c>
-      <x:c r="G7" s="5" t="str">
+      <x:c r="G7" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>TC-7</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>REQ-6</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
+      <x:c r="C8" s="11" t="str">
         <x:v>Payment thành công chuyển Order sang PAID</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="str">
+      <x:c r="D8" s="11" t="str">
         <x:v>Order PAYMENT_PENDING, TotalAmount=100</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="str">
+      <x:c r="E8" s="11" t="str">
         <x:v>Tạo Payment SUCCESS Amount=100</x:v>
       </x:c>
-      <x:c r="F8" s="5" t="str">
+      <x:c r="F8" s="11" t="str">
         <x:v>Tạo đúng một Payment và Order chuyển sang PAID</x:v>
       </x:c>
-      <x:c r="G8" s="5" t="str">
+      <x:c r="G8" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
+      <x:c r="A9" s="11" t="str">
         <x:v>TC-8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
+      <x:c r="B9" s="11" t="str">
         <x:v>REQ-7</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="str">
+      <x:c r="C9" s="11" t="str">
         <x:v>Retry payment có tính idempotent</x:v>
       </x:c>
-      <x:c r="D9" s="5" t="str">
+      <x:c r="D9" s="11" t="str">
         <x:v>Order PAYMENT_PENDING, request có khóa stable-client-request-id</x:v>
       </x:c>
-      <x:c r="E9" s="5" t="str">
+      <x:c r="E9" s="11" t="str">
         <x:v>Gửi cùng request hai lần
 Sau đó thử cùng khóa với Amount khác</x:v>
       </x:c>
-      <x:c r="F9" s="5" t="str">
+      <x:c r="F9" s="11" t="str">
         <x:v>Hai lần đầu trả cùng Payment/TransactionCode và chỉ lưu một bản ghi; Amount khác bị từ chối</x:v>
       </x:c>
-      <x:c r="G9" s="5" t="str">
+      <x:c r="G9" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>TC-9</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B10" s="11" t="str">
         <x:v>REQ-5, REQ-14</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="str">
+      <x:c r="C10" s="11" t="str">
         <x:v>Kiểm chứng mô hình Order kỳ vọng</x:v>
       </x:c>
-      <x:c r="D10" s="5" t="str">
+      <x:c r="D10" s="11" t="str">
         <x:v>order_state_model.json hợp lệ</x:v>
       </x:c>
-      <x:c r="E10" s="5" t="str">
+      <x:c r="E10" s="11" t="str">
         <x:v>Chạy python security-analysis/run_analysis.py</x:v>
       </x:c>
-      <x:c r="F10" s="5" t="str">
+      <x:c r="F10" s="11" t="str">
         <x:v>P1, P2, P3, P4 đều PASS</x:v>
       </x:c>
-      <x:c r="G10" s="5" t="str">
+      <x:c r="G10" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="5" t="str">
+      <x:c r="A11" s="11" t="str">
         <x:v>TC-10</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="str">
+      <x:c r="B11" s="11" t="str">
         <x:v>REQ-5</x:v>
       </x:c>
-      <x:c r="C11" s="5" t="str">
+      <x:c r="C11" s="11" t="str">
         <x:v>Counterexample hồi sinh Order</x:v>
       </x:c>
-      <x:c r="D11" s="5" t="str">
+      <x:c r="D11" s="11" t="str">
         <x:v>order_state_model_buggy.json có cạnh lỗi</x:v>
       </x:c>
-      <x:c r="E11" s="5" t="str">
+      <x:c r="E11" s="11" t="str">
         <x:v>Chạy checker trên model BUGGY</x:v>
       </x:c>
-      <x:c r="F11" s="5" t="str">
+      <x:c r="F11" s="11" t="str">
         <x:v>P1 FAIL với CREATED → CANCELLED → PAID_AFTER_CANCELLED</x:v>
       </x:c>
-      <x:c r="G11" s="5" t="str">
+      <x:c r="G11" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" hidden="0" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+      <x:c r="A12" s="11" t="str">
         <x:v>TC-11</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
+      <x:c r="B12" s="11" t="str">
         <x:v>REQ-9, REQ-10, REQ-11, REQ-12, REQ-13</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="C12" s="11" t="str">
         <x:v>Sanitizer phát hiện đủ 5 bản C lỗi</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="str">
+      <x:c r="D12" s="11" t="str">
         <x:v>GCC, Make, ASan/UBSan khả dụng</x:v>
       </x:c>
-      <x:c r="E12" s="5" t="str">
+      <x:c r="E12" s="11" t="str">
         <x:v>cd security-analysis/c-memory
 make
 make test</x:v>
       </x:c>
-      <x:c r="F12" s="5" t="str">
+      <x:c r="F12" s="11" t="str">
         <x:v>Bản buggy lần lượt báo stack-buffer-overflow, heap-buffer-overflow, heap-use-after-free, memory leak và double-free</x:v>
       </x:c>
-      <x:c r="G12" s="5" t="str">
+      <x:c r="G12" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
-      <x:c r="A13" s="5" t="str">
+      <x:c r="A13" s="11" t="str">
         <x:v>TC-12</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str">
+      <x:c r="B13" s="11" t="str">
         <x:v>REQ-9, REQ-10, REQ-11, REQ-12, REQ-13</x:v>
       </x:c>
-      <x:c r="C13" s="5" t="str">
+      <x:c r="C13" s="11" t="str">
         <x:v>Bản FIXED sạch sanitizer và đúng biên chuỗi</x:v>
       </x:c>
-      <x:c r="D13" s="5" t="str">
+      <x:c r="D13" s="11" t="str">
         <x:v>Đã build cả *_fixed</x:v>
       </x:c>
-      <x:c r="E13" s="5" t="str">
+      <x:c r="E13" s="11" t="str">
         <x:v>Chạy cùng kịch bản lỗi
 Thử Product/User với độ dài 0, 1, 31, 32, 128 byte</x:v>
       </x:c>
-      <x:c r="F13" s="5" t="str">
+      <x:c r="F13" s="11" t="str">
         <x:v>Bản FIXED không có báo cáo sanitizer; nhận tối đa 31 byte và từ chối từ 32 byte; toàn bộ 22/22 case PASS</x:v>
       </x:c>
-      <x:c r="G13" s="5" t="str">
+      <x:c r="G13" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="5" t="str">
+      <x:c r="A14" s="11" t="str">
         <x:v>TC-13</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="str">
+      <x:c r="B14" s="11" t="str">
         <x:v>REQ-4</x:v>
       </x:c>
-      <x:c r="C14" s="5" t="str">
+      <x:c r="C14" s="11" t="str">
         <x:v>Fuzz biên validator Order</x:v>
       </x:c>
-      <x:c r="D14" s="5" t="str">
+      <x:c r="D14" s="11" t="str">
         <x:v>Có xUnit InputValidatorTests</x:v>
       </x:c>
-      <x:c r="E14" s="5" t="str">
+      <x:c r="E14" s="11" t="str">
         <x:v>Chạy các ca null/rỗng, amount, quantity, price, mismatch, nhiều item và giá trị biên</x:v>
       </x:c>
-      <x:c r="F14" s="5" t="str">
+      <x:c r="F14" s="11" t="str">
         <x:v>Input sai bị từ chối; input ở biên hợp lệ được chấp nhận; branch coverage đạt ngưỡng</x:v>
       </x:c>
-      <x:c r="G14" s="5" t="str">
+      <x:c r="G14" s="11" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" hidden="0" customHeight="1">
-      <x:c r="A15" s="5" t="str">
+      <x:c r="A15" s="11" t="str">
         <x:v>TC-14</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="str">
+      <x:c r="B15" s="11" t="str">
         <x:v>REQ-8</x:v>
       </x:c>
-      <x:c r="C15" s="5" t="str">
+      <x:c r="C15" s="11" t="str">
         <x:v>Băm mật khẩu và nâng cấp hash cũ</x:v>
       </x:c>
-      <x:c r="D15" s="5" t="str">
+      <x:c r="D15" s="11" t="str">
         <x:v>Có user mới và user chứa SHA-256 legacy</x:v>
       </x:c>
-      <x:c r="E15" s="5" t="str">
+      <x:c r="E15" s="11" t="str">
         <x:v>Đăng ký user mới
 Đăng nhập user legacy đúng mật khẩu
 Đăng nhập với mật khẩu sai</x:v>
       </x:c>
-      <x:c r="F15" s="5" t="str">
+      <x:c r="F15" s="11" t="str">
         <x:v>Hash mới dùng PasswordHasher; hash legacy được thay bằng hash mới sau lần đăng nhập đúng; mật khẩu sai bị từ chối</x:v>
       </x:c>
-      <x:c r="G15" s="5" t="str">
+      <x:c r="G15" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
-      <x:c r="A16" s="5" t="str">
+      <x:c r="A16" s="11" t="str">
         <x:v>TC-15</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B16" s="11" t="str">
         <x:v>NFR-1</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="str">
+      <x:c r="C16" s="11" t="str">
         <x:v>Rollback khi tạo Order thất bại</x:v>
       </x:c>
-      <x:c r="D16" s="5" t="str">
+      <x:c r="D16" s="11" t="str">
         <x:v>PostgreSQL test database, stock ban đầu đã biết</x:v>
       </x:c>
-      <x:c r="E16" s="5" t="str">
+      <x:c r="E16" s="11" t="str">
         <x:v>Gây lỗi sau khi kiểm tra giá/tồn kho nhưng trước commit
 Đọc lại Order và Product</x:v>
       </x:c>
-      <x:c r="F16" s="5" t="str">
+      <x:c r="F16" s="11" t="str">
         <x:v>Không có Order/OrderItem dở dang; stock không bị giảm một phần</x:v>
       </x:c>
-      <x:c r="G16" s="5" t="str">
+      <x:c r="G16" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
-      <x:c r="A17" s="5" t="str">
+      <x:c r="A17" s="11" t="str">
         <x:v>TC-16</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
+      <x:c r="B17" s="11" t="str">
         <x:v>REQ-15, REQ-16, NFR-6</x:v>
       </x:c>
-      <x:c r="C17" s="5" t="str">
+      <x:c r="C17" s="11" t="str">
         <x:v>Kiểm chứng model phục hồi đầy đủ</x:v>
       </x:c>
-      <x:c r="D17" s="5" t="str">
+      <x:c r="D17" s="11" t="str">
         <x:v>order_payment_recovery_model.json hợp lệ</x:v>
       </x:c>
-      <x:c r="E17" s="5" t="str">
+      <x:c r="E17" s="11" t="str">
         <x:v>Chạy python security-analysis/verify_recovery_model.py
 Đọc 10 thuộc tính và tập state reachable</x:v>
       </x:c>
-      <x:c r="F17" s="5" t="str">
-        <x:v>Model đúng có 14 state, 35 transition; P1-P10 PASS và tất cả state reachable</x:v>
-      </x:c>
-      <x:c r="G17" s="5" t="str">
+      <x:c r="F17" s="11" t="str">
+        <x:v>Model đúng có 14 state, 36 transition; P1-P10 PASS và tất cả state reachable</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
-      <x:c r="A18" s="5" t="str">
+      <x:c r="A18" s="11" t="str">
         <x:v>TC-17</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="str">
+      <x:c r="B18" s="11" t="str">
         <x:v>REQ-5, REQ-15</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="str">
+      <x:c r="C18" s="11" t="str">
         <x:v>Phản ví dụ CANCELLED bị thanh toán</x:v>
       </x:c>
-      <x:c r="D18" s="5" t="str">
+      <x:c r="D18" s="11" t="str">
         <x:v>Mutation BUG-CANCELLED-PAID được bật</x:v>
       </x:c>
-      <x:c r="E18" s="5" t="str">
+      <x:c r="E18" s="11" t="str">
         <x:v>Thêm cạnh CANCELLED → PAID_AFTER_CANCELLED
 Chạy lại toàn bộ thuộc tính</x:v>
       </x:c>
-      <x:c r="F18" s="5" t="str">
+      <x:c r="F18" s="11" t="str">
         <x:v>P1 và P4 FAIL; witness đi từ CREATED tới CANCELLED rồi PAID_AFTER_CANCELLED</x:v>
       </x:c>
-      <x:c r="G18" s="5" t="str">
+      <x:c r="G18" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
-      <x:c r="A19" s="5" t="str">
+      <x:c r="A19" s="11" t="str">
         <x:v>TC-18</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="str">
+      <x:c r="B19" s="11" t="str">
         <x:v>REQ-6, REQ-15</x:v>
       </x:c>
-      <x:c r="C19" s="5" t="str">
+      <x:c r="C19" s="11" t="str">
         <x:v>Phản ví dụ payment sai amount</x:v>
       </x:c>
-      <x:c r="D19" s="5" t="str">
+      <x:c r="D19" s="11" t="str">
         <x:v>Mutation BUG-WRONG-AMOUNT được bật</x:v>
       </x:c>
-      <x:c r="E19" s="5" t="str">
+      <x:c r="E19" s="11" t="str">
         <x:v>Bỏ amount guard tại PAYMENT_PROCESSING
 Chuyển tới PAID_WRONG_AMOUNT</x:v>
       </x:c>
-      <x:c r="F19" s="5" t="str">
+      <x:c r="F19" s="11" t="str">
         <x:v>P1 FAIL và trả witness tới state amount_mismatch</x:v>
       </x:c>
-      <x:c r="G19" s="5" t="str">
+      <x:c r="G19" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
-      <x:c r="A20" s="5" t="str">
+      <x:c r="A20" s="11" t="str">
         <x:v>TC-19</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="str">
+      <x:c r="B20" s="11" t="str">
         <x:v>REQ-7, REQ-18</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="str">
+      <x:c r="C20" s="11" t="str">
         <x:v>Phản ví dụ hai payment SUCCESS</x:v>
       </x:c>
-      <x:c r="D20" s="5" t="str">
+      <x:c r="D20" s="11" t="str">
         <x:v>Mutation BUG-DUPLICATE-SUCCESS được bật</x:v>
       </x:c>
-      <x:c r="E20" s="5" t="str">
+      <x:c r="E20" s="11" t="str">
         <x:v>Bỏ idempotency guard tại PAID
 Tạo state PAID_TWICE</x:v>
       </x:c>
-      <x:c r="F20" s="5" t="str">
+      <x:c r="F20" s="11" t="str">
         <x:v>P1 FAIL và trả witness tới state two_success_payments</x:v>
       </x:c>
-      <x:c r="G20" s="5" t="str">
+      <x:c r="G20" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
-      <x:c r="A21" s="5" t="str">
+      <x:c r="A21" s="11" t="str">
         <x:v>TC-20</x:v>
       </x:c>
-      <x:c r="B21" s="5" t="str">
+      <x:c r="B21" s="11" t="str">
         <x:v>REQ-18, NFR-1</x:v>
       </x:c>
-      <x:c r="C21" s="5" t="str">
+      <x:c r="C21" s="11" t="str">
         <x:v>Phản ví dụ payment-cancel conflict</x:v>
       </x:c>
-      <x:c r="D21" s="5" t="str">
+      <x:c r="D21" s="11" t="str">
         <x:v>Mutation BUG-RESOURCE-CONFLICT được bật</x:v>
       </x:c>
-      <x:c r="E21" s="5" t="str">
+      <x:c r="E21" s="11" t="str">
         <x:v>Cho payment và cancel cùng sở hữu resource
 Chạy kiểm chứng</x:v>
       </x:c>
-      <x:c r="F21" s="5" t="str">
+      <x:c r="F21" s="11" t="str">
         <x:v>P1 và P7 FAIL với witness tới PAY_CANCEL_CONFLICT</x:v>
       </x:c>
-      <x:c r="G21" s="5" t="str">
+      <x:c r="G21" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
-      <x:c r="A22" s="5" t="str">
+      <x:c r="A22" s="11" t="str">
         <x:v>TC-21</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="str">
+      <x:c r="B22" s="11" t="str">
         <x:v>REQ-16, REQ-17</x:v>
       </x:c>
-      <x:c r="C22" s="5" t="str">
+      <x:c r="C22" s="11" t="str">
         <x:v>Bounded retry và compensation</x:v>
       </x:c>
-      <x:c r="D22" s="5" t="str">
+      <x:c r="D22" s="11" t="str">
         <x:v>Model đúng, weak fairness được khai báo</x:v>
       </x:c>
-      <x:c r="E22" s="5" t="str">
+      <x:c r="E22" s="11" t="str">
         <x:v>Đi PAYMENT_PROCESSING → PAYMENT_RETRY → PAYMENT_PROCESSING_FINAL
 Thử timeout cuối và charged-but-commit-failed</x:v>
       </x:c>
-      <x:c r="F22" s="5" t="str">
+      <x:c r="F22" s="11" t="str">
         <x:v>Không có vòng retry tiến triển vô hạn; nhánh cuối tới FAILED hoặc REFUND_PENDING → REFUNDED</x:v>
       </x:c>
-      <x:c r="G22" s="5" t="str">
+      <x:c r="G22" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="66" customHeight="1">
+      <x:c r="A23" s="13" t="str">
+        <x:v>TC-22</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>REQ-15, NFR-6</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>Nạp workbook bằng pipeline Spec Verification Lab</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>Python 3.14, openpyxl và z3-solver khả dụng</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>Gọi parse_specification_excel() trên workbook
+Chạy run_pipeline(..., fuzz_iterations=300, seed=1)
+Đọc báo cáo bốn chương</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>Nạp đủ 10 sheet; không deadlock; toàn bộ công thức CTL hợp lệ báo DUNG; mutual exclusion OK; pipeline hoàn tất không exception</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="66" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>TC-23</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>REQ-18, REQ-22, NFR-1, NFR-7</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>Race payment và cancellation trên PostgreSQL</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>Docker hoạt động; PostgreSQL Testcontainer sạch; Order PAYMENT_PENDING</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>Gửi POST /api/payments và POST /api/orders/{id}/cancel đồng thời
+Đọc lại Order, Payment và InventoryStatus</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>Chỉ một thao tác thắng; kết quả cuối chỉ là PAID + SUCCESS + RESERVED hoặc CANCELLED + không Payment + RELEASED</x:v>
+      </x:c>
+      <x:c r="G24" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="66" customHeight="1">
+      <x:c r="A25" s="13" t="str">
+        <x:v>TC-24</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>REQ-19, REQ-23, NFR-8</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>Worker reconcile Payment UNKNOWN sau restart</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>Payment UNKNOWN/PROCESSING đã stale; gateway lưu kết quả theo idempotency key</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="str">
+        <x:v>Khởi động worker với ngưỡng stale đã đạt
+Chờ một chu kỳ quét
+Đọc Payment và Order</x:v>
+      </x:c>
+      <x:c r="F25" s="14" t="str">
+        <x:v>Worker chỉ gọi status query, không charge lần hai; kết quả được finalize hoặc giữ UNKNOWN để lần quét sau xử lý</x:v>
+      </x:c>
+      <x:c r="G25" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="66" customHeight="1">
+      <x:c r="A26" s="13" t="str">
+        <x:v>TC-25</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>REQ-20, REQ-24</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>Inventory chuyển RELEASED hoặc CONSUMED đúng một lần</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>Có Order với inventory RESERVED</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>Hủy một Order chưa charge và gọi hủy lại
+Thanh toán Order khác, Admin confirm rồi complete và gọi complete lại</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>Order hủy có RELEASED và stock chỉ hoàn một lần; Order hoàn tất có CONSUMED và không hoàn stock</x:v>
+      </x:c>
+      <x:c r="G26" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="66" customHeight="1">
+      <x:c r="A27" s="13" t="str">
+        <x:v>TC-26</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>REQ-17, REQ-21</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>Refund idempotent và reconcile sau crash</x:v>
+      </x:c>
+      <x:c r="D27" s="14" t="str">
+        <x:v>Admin JWT; Payment SUCCESS; Order PAID hoặc CONFIRMED</x:v>
+      </x:c>
+      <x:c r="E27" s="14" t="str">
+        <x:v>POST refund với key ổn định
+Lặp request cùng key
+Mô phỏng crash trước finalize rồi gọi refund/reconcile</x:v>
+      </x:c>
+      <x:c r="F27" s="14" t="str">
+        <x:v>Chỉ một refund gateway; Payment/Order đi REFUND_PENDING → REFUNDED; inventory RELEASED đúng một lần</x:v>
+      </x:c>
+      <x:c r="G27" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="66" customHeight="1">
+      <x:c r="A28" s="13" t="str">
+        <x:v>TC-27</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>REQ-7, REQ-22</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>Hai yêu cầu payment đồng thời</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>PostgreSQL Testcontainer; một Order PAYMENT_PENDING</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>Gửi hai POST /api/payments với hai key khác nhau cùng lúc
+Đọc bảng Payments</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>Một request HTTP 201, request còn lại HTTP 409; database chỉ có một Payment SUCCESS cho Order</x:v>
+      </x:c>
+      <x:c r="G28" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="66" customHeight="1">
+      <x:c r="A29" s="13" t="str">
+        <x:v>TC-28</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>REQ-24</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>Phân quyền và chuỗi confirm-complete</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>Customer có Order PAID; có JWT Customer và Admin</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="str">
+        <x:v>Customer gọi confirm/complete
+Admin gọi confirm
+Admin gọi complete</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>Customer nhận 403; Admin nhận PAID → CONFIRMED → COMPLETED và InventoryStatus=CONSUMED</x:v>
+      </x:c>
+      <x:c r="G29" s="13" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
@@ -937,254 +1124,338 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>REQ-1</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>Mọi API Cart, Order và Payment phải yêu cầu JWT hợp lệ; chỉ Admin được liệt kê toàn bộ đơn hàng.</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
-        <x:v>authentication</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>REQ-2</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>Người dùng chỉ được đọc hoặc thay đổi User, Cart, Order và Payment thuộc chính mình; quyền Admin là ngoại lệ được kiểm soát.</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
-        <x:v>authorization</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>REQ-3</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>Khi tạo đơn, giá sản phẩm phải lấy từ cơ sở dữ liệu phía server, sản phẩm phải tồn tại/đang hoạt động và tồn kho phải đủ.</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>integrity</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="str">
+      <x:c r="C4" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>REQ-4</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>TotalAmount phải dương, trong giới hạn cho phép và khớp tổng Quantity × UnitPrice với sai số tối đa 0,01; dữ liệu sai phải bị từ chối.</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
-        <x:v>validation</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="C5" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>REQ-5</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>Order chỉ được chuyển theo chuỗi CREATED → VALIDATED → PAYMENT_PENDING → PAID → CONFIRMED → COMPLETED; không bỏ bước, quay ngược hoặc hồi sinh trạng thái terminal.</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>safety</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>REQ-6</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>Order chỉ được chuyển từ PAYMENT_PENDING sang PAID khi có Payment SUCCESS với Amount đúng bằng Order.TotalAmount.</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
-        <x:v>consistency</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>REQ-7</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>Mỗi yêu cầu thanh toán phải có IdempotencyKey; gửi lại cùng khóa và cùng Amount phải trả về giao dịch cũ, còn tái dùng khóa với Amount khác phải bị từ chối.</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
-        <x:v>payment</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="str">
+      <x:c r="C8" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
+      <x:c r="A9" s="11" t="str">
         <x:v>REQ-8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
+      <x:c r="B9" s="11" t="str">
         <x:v>Mật khẩu mới phải được băm bằng PasswordHasher có salt/work factor; tài khoản SHA-256 cũ chỉ được xác minh để nâng cấp một lần.</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>credential</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
+      <x:c r="C9" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>REQ-9</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B10" s="11" t="str">
         <x:v>register_user() không được sao chép email dài từ 32 byte trở lên vào buffer stack 32 byte.</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="str">
+      <x:c r="C10" s="11" t="str">
         <x:v>memory</x:v>
       </x:c>
-      <x:c r="D10" s="5" t="str">
+      <x:c r="D10" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="5" t="str">
+      <x:c r="A11" s="11" t="str">
         <x:v>REQ-10</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="str">
+      <x:c r="B11" s="11" t="str">
         <x:v>Product name không được vượt biên buffer heap 32 byte; nhánh từ chối vẫn phải giải phóng vùng nhớ đã cấp phát.</x:v>
       </x:c>
-      <x:c r="C11" s="5" t="str">
+      <x:c r="C11" s="11" t="str">
         <x:v>memory</x:v>
       </x:c>
-      <x:c r="D11" s="5" t="str">
+      <x:c r="D11" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+      <x:c r="A12" s="11" t="str">
         <x:v>REQ-11</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
+      <x:c r="B12" s="11" t="str">
         <x:v>Cart audit log không được đọc CartItem sau khi phần tử đã được free.</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="C12" s="11" t="str">
         <x:v>memory</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="str">
+      <x:c r="D12" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="5" t="str">
+      <x:c r="A13" s="11" t="str">
         <x:v>REQ-12</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str">
+      <x:c r="B13" s="11" t="str">
         <x:v>Khi hủy Order trong mô hình C, mảng OrderItem thuộc sở hữu của Order phải được free trước struct cha.</x:v>
       </x:c>
-      <x:c r="C13" s="5" t="str">
+      <x:c r="C13" s="11" t="str">
         <x:v>memory</x:v>
       </x:c>
-      <x:c r="D13" s="5" t="str">
+      <x:c r="D13" s="11" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="5" t="str">
+      <x:c r="A14" s="11" t="str">
         <x:v>REQ-13</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="str">
+      <x:c r="B14" s="11" t="str">
         <x:v>Payment cleanup không được free TransactionCode hai lần; con trỏ sở hữu phải được đặt NULL sau lần free đầu.</x:v>
       </x:c>
-      <x:c r="C14" s="5" t="str">
+      <x:c r="C14" s="11" t="str">
         <x:v>memory</x:v>
       </x:c>
-      <x:c r="D14" s="5" t="str">
+      <x:c r="D14" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
-      <x:c r="A15" s="5" t="str">
+      <x:c r="A15" s="11" t="str">
         <x:v>REQ-14</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="str">
-        <x:v>Từ mọi trạng thái Order có thể đạt tới, mọi đường thực thi hữu hạn tiến triển phải cuối cùng tới COMPLETED, CANCELLED hoặc FAILED.</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="str">
+      <x:c r="B15" s="11" t="str">
+        <x:v>Từ mọi trạng thái Order có thể đạt tới, mọi đường tiến triển phải cuối cùng tới COMPLETED, CANCELLED, FAILED hoặc REFUNDED.</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
         <x:v>liveness</x:v>
       </x:c>
-      <x:c r="D15" s="5" t="str">
+      <x:c r="D15" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
-      <x:c r="A16" s="5" t="str">
+      <x:c r="A16" s="11" t="str">
         <x:v>REQ-15</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B16" s="11" t="str">
         <x:v>Mỗi trạng thái Order-Payment phải đặc tả sự cố, cách phát hiện, biện pháp xử lý và trạng thái tiếp theo; không được có sự cố không có đường phục hồi hoặc kết thúc.</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="str">
+      <x:c r="C16" s="11" t="str">
         <x:v>safety</x:v>
       </x:c>
-      <x:c r="D16" s="5" t="str">
+      <x:c r="D16" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
-      <x:c r="A17" s="5" t="str">
+      <x:c r="A17" s="11" t="str">
         <x:v>REQ-16</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
-        <x:v>Retry thanh toán và xác nhận phải có bound; khi hết ngân sách retry phải chuyển FAILED hoặc REFUND_PENDING thay vì lặp vô hạn.</x:v>
-      </x:c>
-      <x:c r="C17" s="5" t="str">
+      <x:c r="B17" s="11" t="str">
+        <x:v>Charge có tối đa hai attempt (lần đầu và một retry). Khi hết ngân sách không được charge lại; hệ thống chỉ reconcile cho tới khi biết kết quả PAID, FAILED hoặc chuyển sang refund compensation.</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="str">
         <x:v>liveness</x:v>
       </x:c>
-      <x:c r="D17" s="5" t="str">
+      <x:c r="D17" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
-      <x:c r="A18" s="5" t="str">
+      <x:c r="A18" s="11" t="str">
         <x:v>REQ-17</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="str">
+      <x:c r="B18" s="11" t="str">
         <x:v>Nếu gateway đã charge nhưng không thể hoàn tất đơn hoặc commit PAID, hệ thống phải dùng REFUND_PENDING và REFUNDED để bù trừ; không được đổi thẳng sang FAILED.</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="str">
-        <x:v>consistency</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="str">
+      <x:c r="C18" s="11" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
-      <x:c r="A19" s="5" t="str">
+      <x:c r="A19" s="11" t="str">
         <x:v>REQ-18</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="str">
+      <x:c r="B19" s="11" t="str">
         <x:v>Payment và cancellation trên cùng Order phải được serialize; không được đồng thời sở hữu critical resource hoặc tạo hai Payment SUCCESS.</x:v>
       </x:c>
-      <x:c r="C19" s="5" t="str">
+      <x:c r="C19" s="11" t="str">
         <x:v>safety</x:v>
       </x:c>
-      <x:c r="D19" s="5" t="str">
+      <x:c r="D19" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="13" t="str">
+        <x:v>REQ-19</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Worker phục hồi phải quét Payment PROCESSING, UNKNOWN và REFUND_PENDING đã quá hạn; chỉ truy vấn trạng thái gateway, không được tạo charge mới.</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>liveness</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="13" t="str">
+        <x:v>REQ-20</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>Inventory reservation phải được RELEASED đúng một lần khi Order CANCELLED, FAILED hoặc REFUNDED và được CONSUMED đúng một lần khi Order COMPLETED.</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="13" t="str">
+        <x:v>REQ-21</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>Chỉ Admin được khởi tạo/retry/reconcile refund; refund dùng idempotency key riêng và callback lặp không được hoàn tiền lần hai.</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="13" t="str">
+        <x:v>REQ-22</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>Order, Payment và Product phải phát hiện cập nhật cạnh tranh bằng concurrency token hoặc ràng buộc database và trả HTTP 409 cho xung đột có thể retry.</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>REQ-23</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>Gateway timeout hoặc exception phải đưa Payment về UNKNOWN; hệ thống không được suy diễn UNKNOWN là FAILED và không được hoàn kho trước khi reconcile.</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>safety</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="13" t="str">
+        <x:v>REQ-24</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Chỉ Admin được chuyển Order PAID sang CONFIRMED và CONFIRMED sang COMPLETED; hoàn tất phải consume inventory reservation.</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>functional</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
@@ -1214,68 +1485,101 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>NFR-1</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>Các thay đổi Order, tồn kho và Payment phải được lưu nguyên tử; luồng dùng PostgreSQL phải chạy trong transaction mức Serializable.</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>NFR-2</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>Branch coverage của lớp kiểm tra đầu vào và các guard trạng thái trọng yếu phải đạt tối thiểu 90% trong pipeline kiểm thử.</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>NFR-3</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>Log lỗi phải đủ OrderId/UserId để truy vết nhưng không được ghi mật khẩu, JWT, Jwt:Key hoặc connection string.</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="C4" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>NFR-4</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>Secret và connection string phải được cung cấp ngoài source control; Jwt:Key phải có ít nhất 32 ký tự.</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>NFR-5</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>Các bản C biên dịch với AddressSanitizer/UndefinedBehaviorSanitizer phải phát hiện đúng bản lỗi và không báo lỗi với bản FIXED trên cùng ca kiểm thử.</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>NFR-6</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>Pipeline kiểm chứng phải duyệt toàn bộ model hữu hạn, lưu counterexample cho model lỗi và ghi rõ bound, fairness, assumptions và giới hạn kết luận.</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="13" t="str">
+        <x:v>NFR-7</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>Bộ kiểm thử phải tái lập được trên PostgreSQL sạch bằng Testcontainers và không được dùng database phát triển.</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="13" t="str">
+        <x:v>NFR-8</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>Recovery worker phải cấu hình được chu kỳ quét, ngưỡng stale và batch size; một lỗi đơn lẻ không được dừng các lần quét sau.</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="13" t="str">
+        <x:v>NFR-9</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>Payment gateway call phải chạy ngoài database transaction để không giữ khóa trong thời gian chờ mạng.</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
         <x:v>HIGH</x:v>
       </x:c>
     </x:row>
@@ -1303,107 +1607,139 @@
       <x:c r="C1" s="10" t="str">
         <x:v>MucUuTien</x:v>
       </x:c>
+      <x:c r="D1" s="13"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>CON-1</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>Ứng dụng dùng ASP.NET Core/.NET 10, Entity Framework Core và PostgreSQL; API trao đổi JSON qua REST.</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
+      <x:c r="D2" s="13"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>CON-2</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>Order/Payment Amount nằm trong [0,01; 999999,99], Quantity nằm trong [1; 10000], và UnitPrice nằm trong [0,01; 999999,99].</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
-      <x:c r="D3"/>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D3" s="13"/>
+    </x:row>
+    <x:row r="4" ht="34" hidden="0" customHeight="1">
+      <x:c r="A4" s="11" t="str">
         <x:v>CON-3</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>IdempotencyKey bắt buộc, không trắng và dài tối đa 128 ký tự; khóa là duy nhất trong phạm vi một Order.</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
-      <x:c r="D4"/>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
+        <x:v>IdempotencyKey bắt buộc, không trắng, dài tối đa 128 ký tự và duy nhất toàn hệ thống cho một logical charge; RefundIdempotencyKey là khóa riêng.</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D4" s="13"/>
+    </x:row>
+    <x:row r="5" ht="34" hidden="0" customHeight="1">
+      <x:c r="A5" s="11" t="str">
         <x:v>CON-4</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
-        <x:v>Order terminal gồm COMPLETED, CANCELLED và FAILED; mô hình Kripke dùng self-loop ở trạng thái terminal để quan hệ chuyển là total.</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Order terminal gồm COMPLETED, CANCELLED, FAILED và REFUNDED; mỗi trạng thái terminal có self-loop để quan hệ chuyển là total.</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D5" s="13"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>CON-5</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>Buffer email và product name trong mô hình C có 32 byte, nên chuỗi hợp lệ dài tối đa 31 byte để dành chỗ cho NUL.</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D6" s="13"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>CON-6</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>Năm mô-đun C là mô hình học tập về ownership/lifetime, không phải bằng chứng rằng ứng dụng C# managed mắc cùng lỗi bộ nhớ.</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
         <x:v>MEDIUM</x:v>
       </x:c>
+      <x:c r="D7" s="13"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>CON-7</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>Model dùng tối đa một lần retry thanh toán cuối; PAYMENT_PROCESSING_FINAL không được quay lại PAYMENT_RETRY.</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="24" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
+      <x:c r="C8" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D8" s="13"/>
+    </x:row>
+    <x:row r="9" ht="34" hidden="0" customHeight="1">
+      <x:c r="A9" s="11" t="str">
         <x:v>CON-8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>Thuộc tính liveness dùng weak fairness: cạnh no-op/retry được đánh dấu stutter có thể lặp, nhưng transition tiến triển đang enable cuối cùng phải chạy.</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Recovery model JSON dùng weak fairness cho cạnh stutter; mô hình Excel dùng cho checker CTL cơ bản loại bỏ self-loop ở trạng thái chưa terminal để kiểm tra AF(terminal).</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D9" s="13"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>CON-9</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B10" s="11" t="str">
         <x:v>Refund dùng idempotency key riêng; callback refund trùng chỉ trả kết quả đã lưu và không hoàn tiền lần hai.</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="str">
-        <x:v>HIGH</x:v>
-      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D10" s="13"/>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="13" t="str">
+        <x:v>CON-10</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>Một logical Payment duy nhất cho mỗi Order; charge có tối đa 2 attempt và mọi retry phải dùng lại idempotency key ban đầu.</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D11" s="13"/>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="13" t="str">
+        <x:v>CON-11</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>Gateway charge/refund chạy ngoài transaction; database chỉ lưu intent trước call và finalize/reconcile kết quả trong lần ghi riêng.</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D12" s="13"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1435,172 +1771,172 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>CREATED</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>x</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>created, inventory_unreserved</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="11" t="str">
         <x:v>VALIDATED, FAILED</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>VALIDATED</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str"/>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="B3" s="11" t="str"/>
+      <x:c r="C3" s="11" t="str">
         <x:v>validated, inventory_reserved, amount_verified</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="D3" s="11" t="str">
         <x:v>PAYMENT_PENDING, FAILED</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>PAYMENT_PENDING</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str"/>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="B4" s="11" t="str"/>
+      <x:c r="C4" s="11" t="str">
         <x:v>payment_pending, inventory_reserved, amount_verified</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str">
-        <x:v>PAYMENT_PROCESSING, CANCELLED, PAYMENT_PENDING</x:v>
+      <x:c r="D4" s="11" t="str">
+        <x:v>PAYMENT_PROCESSING, CANCELLED</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>PAYMENT_PROCESSING</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str"/>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="B5" s="11" t="str"/>
+      <x:c r="C5" s="11" t="str">
         <x:v>payment_processing, inventory_reserved, amount_verified, payment_lock</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
-        <x:v>PAID, PAYMENT_RETRY, FAILED, REFUND_PENDING, PAYMENT_PROCESSING</x:v>
+      <x:c r="D5" s="11" t="str">
+        <x:v>PAID, PAYMENT_RETRY, FAILED, REFUND_PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>PAYMENT_RETRY</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str"/>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="B6" s="11" t="str"/>
+      <x:c r="C6" s="11" t="str">
         <x:v>payment_retry, inventory_reserved, amount_verified</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>PAYMENT_PROCESSING_FINAL, FAILED, CANCELLED</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>PAYMENT_PROCESSING_FINAL</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str"/>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="B7" s="11" t="str"/>
+      <x:c r="C7" s="11" t="str">
         <x:v>payment_processing, final_retry, inventory_reserved, amount_verified, payment_lock</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="11" t="str">
         <x:v>PAID, FAILED, REFUND_PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>PAID</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str"/>
-      <x:c r="C8" s="5" t="str">
+      <x:c r="B8" s="11" t="str"/>
+      <x:c r="C8" s="11" t="str">
         <x:v>paid, payment_success, amount_verified, inventory_reserved</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="str">
-        <x:v>CONFIRMED, PAID, CONFIRMATION_RETRY, REFUND_PENDING</x:v>
+      <x:c r="D8" s="11" t="str">
+        <x:v>CONFIRMED, CONFIRMATION_RETRY, REFUND_PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
+      <x:c r="A9" s="11" t="str">
         <x:v>CONFIRMATION_RETRY</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str"/>
-      <x:c r="C9" s="5" t="str">
+      <x:c r="B9" s="11" t="str"/>
+      <x:c r="C9" s="11" t="str">
         <x:v>paid, payment_success, confirmation_retry, amount_verified</x:v>
       </x:c>
-      <x:c r="D9" s="5" t="str">
+      <x:c r="D9" s="11" t="str">
         <x:v>CONFIRMED, REFUND_PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str"/>
-      <x:c r="C10" s="5" t="str">
+      <x:c r="B10" s="11" t="str"/>
+      <x:c r="C10" s="11" t="str">
         <x:v>confirmed, paid, payment_success, amount_verified</x:v>
       </x:c>
-      <x:c r="D10" s="5" t="str">
+      <x:c r="D10" s="11" t="str">
         <x:v>COMPLETED, REFUND_PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="5" t="str">
+      <x:c r="A11" s="11" t="str">
         <x:v>REFUND_PENDING</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="str"/>
-      <x:c r="C11" s="5" t="str">
+      <x:c r="B11" s="11" t="str"/>
+      <x:c r="C11" s="11" t="str">
         <x:v>paid, payment_success, refund_pending, amount_verified</x:v>
       </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>REFUNDED, REFUND_PENDING</x:v>
+      <x:c r="D11" s="11" t="str">
+        <x:v>REFUNDED</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+      <x:c r="A12" s="11" t="str">
         <x:v>COMPLETED</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str"/>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="B12" s="11" t="str"/>
+      <x:c r="C12" s="11" t="str">
         <x:v>completed, paid, payment_success, amount_verified, terminal</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="str">
+      <x:c r="D12" s="11" t="str">
         <x:v>COMPLETED</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="5" t="str">
+      <x:c r="A13" s="11" t="str">
         <x:v>CANCELLED</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str"/>
-      <x:c r="C13" s="5" t="str">
+      <x:c r="B13" s="11" t="str"/>
+      <x:c r="C13" s="11" t="str">
         <x:v>cancelled, inventory_released, terminal</x:v>
       </x:c>
-      <x:c r="D13" s="5" t="str">
+      <x:c r="D13" s="11" t="str">
         <x:v>CANCELLED</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="5" t="str">
+      <x:c r="A14" s="11" t="str">
         <x:v>FAILED</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="str"/>
-      <x:c r="C14" s="5" t="str">
+      <x:c r="B14" s="11" t="str"/>
+      <x:c r="C14" s="11" t="str">
         <x:v>failed, inventory_released, terminal</x:v>
       </x:c>
-      <x:c r="D14" s="5" t="str">
+      <x:c r="D14" s="11" t="str">
         <x:v>FAILED</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="5" t="str">
+      <x:c r="A15" s="11" t="str">
         <x:v>REFUNDED</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="str"/>
-      <x:c r="C15" s="5" t="str">
+      <x:c r="B15" s="11" t="str"/>
+      <x:c r="C15" s="11" t="str">
         <x:v>refunded, payment_compensated, inventory_released, terminal</x:v>
       </x:c>
-      <x:c r="D15" s="5" t="str">
+      <x:c r="D15" s="11" t="str">
         <x:v>REFUNDED</x:v>
       </x:c>
     </x:row>
@@ -1622,53 +1958,78 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>AG(!violation)</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
-        <x:v>AG(paid -&gt; payment_success)</x:v>
+      <x:c r="A3" s="11" t="str">
+        <x:v>AG(!resource_conflict)</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>AG(completed -&gt; payment_success)</x:v>
+      <x:c r="A4" s="11" t="str">
+        <x:v>EF(payment_pending)</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
-        <x:v>AG(cancelled -&gt; !payment_success)</x:v>
+      <x:c r="A5" s="11" t="str">
+        <x:v>EF(payment_processing)</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
-        <x:v>AG(failed -&gt; !payment_success)</x:v>
+      <x:c r="A6" s="11" t="str">
+        <x:v>EF(payment_lock)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
-        <x:v>AG(payment_pending -&gt; !payment_success)</x:v>
+      <x:c r="A7" s="11" t="str">
+        <x:v>EF(paid)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
-        <x:v>AG(!resource_conflict)</x:v>
+      <x:c r="A8" s="11" t="str">
+        <x:v>EF(payment_success)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
-        <x:v>AG(refund_pending -&gt; payment_success)</x:v>
+      <x:c r="A9" s="11" t="str">
+        <x:v>EF(completed)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="5" t="str">
-        <x:v>AG(refunded -&gt; payment_compensated)</x:v>
+      <x:c r="A10" s="11" t="str">
+        <x:v>EF(cancelled)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="5" t="str">
-        <x:v>AG(payment_processing -&gt; AF(terminal))</x:v>
+      <x:c r="A11" s="11" t="str">
+        <x:v>EF(failed)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>EF(refund_pending)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>EF(refunded)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>EF(payment_compensated)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>EF(terminal)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>AF(terminal)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1694,66 +2055,66 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
-        <x:v>payment_pending</x:v>
-      </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
+        <x:v>payment_lock</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str">
+        <x:v>cancelled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>cancelled</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
         <x:v>payment_success</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
-        <x:v>cancelled</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="str">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="11" t="str">
+        <x:v>failed</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
         <x:v>payment_success</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>failed</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>payment_success</x:v>
-      </x:c>
-    </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>resource_conflict</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>payment_lock</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>resource_conflict</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>cancel_lock</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>two_success_payments</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>safe</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>amount_mismatch</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>amount_verified</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="5" t="str">
+      <x:c r="A9" s="11" t="str">
         <x:v>refunded</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
+      <x:c r="B9" s="11" t="str">
         <x:v>refund_pending</x:v>
       </x:c>
     </x:row>
@@ -1804,184 +2165,184 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>register_user</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>c</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>buffer_copy</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="11" t="str">
         <x:v>input</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="n">
+      <x:c r="E2" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F2" s="5" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>buffer-overflow</x:v>
       </x:c>
-      <x:c r="G2" s="5" t="n">
+      <x:c r="G2" s="11" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="H2" s="5" t="n">
+      <x:c r="H2" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>import_product_name</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>c</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
         <x:v>buffer_copy</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="D3" s="11" t="str">
         <x:v>input</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="n">
+      <x:c r="E3" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F3" s="5" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>buffer-overflow</x:v>
       </x:c>
-      <x:c r="G3" s="5" t="n">
+      <x:c r="G3" s="11" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="H3" s="5" t="n">
+      <x:c r="H3" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>remove_cart_item</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>c</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="C4" s="11" t="str">
         <x:v>alloc_release</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str">
+      <x:c r="D4" s="11" t="str">
         <x:v>removed</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="n">
+      <x:c r="E4" s="11" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>use-after-free</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="n">
+      <x:c r="G4" s="11" t="n">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="n">
+      <x:c r="H4" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>cancel_order</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>c</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>alloc_release</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>order, order-&gt;items</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="n">
+      <x:c r="E5" s="11" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="F5" s="5" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>memory-leak</x:v>
       </x:c>
-      <x:c r="G5" s="5" t="n">
+      <x:c r="G5" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H5" s="5" t="n">
+      <x:c r="H5" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>cleanup_payment</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>c</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>alloc_release</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>transaction_code</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="n">
+      <x:c r="E6" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F6" s="5" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>double-free</x:v>
       </x:c>
-      <x:c r="G6" s="5" t="n">
+      <x:c r="G6" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H6" s="5" t="n">
+      <x:c r="H6" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>safe_divide_retry_budget</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>python</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
         <x:v>divide</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="11" t="str">
         <x:v>remaining_attempts, elapsed_ms</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="n">
+      <x:c r="E7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F7" s="5" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>divide-by-zero</x:v>
       </x:c>
-      <x:c r="G7" s="5" t="n">
+      <x:c r="G7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H7" s="5" t="n">
+      <x:c r="H7" s="11" t="n">
         <x:v>1000</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="5" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>verify_gateway_callback</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>python</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
+      <x:c r="C8" s="11" t="str">
         <x:v>magic_value</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="str">
+      <x:c r="D8" s="11" t="str">
         <x:v>signature_code</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="n">
+      <x:c r="E8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F8" s="5" t="str">
+      <x:c r="F8" s="11" t="str">
         <x:v>authentication-bypass</x:v>
       </x:c>
-      <x:c r="G8" s="5" t="n">
+      <x:c r="G8" s="11" t="n">
         <x:v>4919</x:v>
       </x:c>
-      <x:c r="H8" s="5" t="n">
+      <x:c r="H8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2015,86 +2376,86 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="11" t="str">
         <x:v>order_item_subtotal_cents</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B2" s="11" t="str">
         <x:v>quantity, unit_price_cents</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="C2" s="11" t="str">
         <x:v>1 &lt;= quantity &lt;= 10000 and 1 &lt;= unit_price_cents &lt;= 99999999 and quantity * unit_price_cents &gt; 2147483647</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="11" t="str">
         <x:v>quantity * unit_price_cents</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="11" t="str">
         <x:v>order_total_cents</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="11" t="str">
         <x:v>subtotal1, subtotal2</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="C3" s="11" t="str">
         <x:v>subtotal1 &gt;= 0 and subtotal2 &gt;= 0 and subtotal1 + subtotal2 &gt; 2147483647</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="D3" s="11" t="str">
         <x:v>subtotal1 + subtotal2</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>two_payment_total_cents</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>payment1_cents, payment2_cents</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="C4" s="11" t="str">
         <x:v>payment1_cents &gt;= 0 and payment2_cents &gt;= 0 and payment1_cents + payment2_cents &gt; 2147483647</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str">
+      <x:c r="D4" s="11" t="str">
         <x:v>payment1_cents + payment2_cents</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>inventory_after_reserve</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>stock, quantity</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>0 &lt;= stock &lt;= 2147483647 and 1 &lt;= quantity &lt;= 10000 and stock - quantity &lt; 0</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>stock - quantity</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="5" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>retry_counter_increment</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>retry_count, one</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="11" t="str">
         <x:v>0 &lt;= retry_count &lt;= 2147483647 and one == 1 and retry_count + one &gt; 2147483647</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="11" t="str">
         <x:v>retry_count + one</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="5" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>refund_total_cents</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>paid_cents, refunded_cents</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="11" t="str">
         <x:v>paid_cents &gt;= 0 and refunded_cents &gt;= 0 and paid_cents + refunded_cents &gt; 2147483647</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="11" t="str">
         <x:v>paid_cents + refunded_cents</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
yêu cầu bảo mật Order–Payment, mô hình trạng thái, thuộc tính CTL, kiểm tra số học, 5 mô-đun lỗi bộ nhớ C và 15 test case. File đã được kiểm tra hợp lệ OpenXML
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -455,7 +455,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="43.2" customHeight="1">
+    <row r="3" ht="57.6" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>description</t>
@@ -463,7 +463,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Đặc tả kiểm chứng hình thức cho luồng Order-Payment: state machine có xử lý sự cố và phục hồi, safety/liveness, idempotency, serialization payment-cancel, bounded retry, compensation refund, SMT số học và mô hình C về an toàn bộ nhớ.</t>
+          <t>Đặc tả kiểm chứng hình thức cho luồng Order-Payment: state machine có xử lý sự cố và phục hồi, safety/liveness, idempotency, serialization payment-cancel, bounded retry, compensation refund, SMT số học, fuzzing xác định, TLC, integration PostgreSQL và mô hình C về an toàn bộ nhớ.</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1" style="1"/>
@@ -1425,6 +1425,154 @@
         </is>
       </c>
       <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28.8" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>TC-25</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-2, REQ-7, REQ-18, NFR-1</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>Integration HTTP với PostgreSQL thật</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Docker hoặc PostgreSQL binaries cục bộ khả dụng</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Chạy dotnet test cho OrderPaymentMicroservice.IntegrationTests</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>5/5 PASS: xác thực/quyền sở hữu, rollback, idempotency, payment-cancel và concurrency được kiểm tra trên PostgreSQL</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28.8" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>TC-26</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>REQ-4, REQ-5, REQ-6, NFR-2</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>Fuzzing xác định validator và state machine</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Có corpus, seed cố định, timeout và crash policy</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python security-analysis/run_fuzzing.py</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>3/3 campaign PASS; 25.000 iteration cho validator và 25.000 transition; branch coverage 99,07%, không crash</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28.8" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>TC-27</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>REQ-5, REQ-14, REQ-16, REQ-17, NFR-6</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>TLC kiểm chứng đặc tả TLA+</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>Có tla2tools.jar</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python security-analysis/run_tlc.py --jar /duong-dan/tla2tools.jar</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>TLC không phát hiện lỗi: 35 state sinh, 20 state phân biệt, độ sâu 9; safety và liveness đều thỏa</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28.8" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>TC-28</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>REQ-5, REQ-14, NFR-6</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>Tương thích bộ công cụ ATPM của giảng viên</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>Workbook và JSON pipeline đã sinh</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>Chạy pytest ATPM/atpm_project/python/tests/test_order_payment_spec.py và verify_teacher_spec.py</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>Schema đúng 10 sheet; Excel/JSON đồng nghĩa; Kripke total và reachable; 7/7 CTL PASS; 6/6 test đặc tả PASS</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1485,7 +1633,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>authentication</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -1507,7 +1655,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>authorization</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -1529,7 +1677,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>integrity</t>
+          <t>functional</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -1551,7 +1699,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1595,7 +1743,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>consistency</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -1617,7 +1765,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>functional</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -1639,7 +1787,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>credential</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -1837,7 +1985,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>consistency</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -2250,7 +2398,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>created, inventory_unreserved</t>
+          <t>created, inventory_unreserved, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2272,7 +2420,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>validated, inventory_reserved, amount_verified</t>
+          <t>validated, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2294,7 +2442,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>payment_pending, inventory_reserved, amount_verified</t>
+          <t>payment_pending, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2316,7 +2464,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>payment_processing, inventory_reserved, amount_verified, payment_lock</t>
+          <t>payment_processing, inventory_reserved, amount_verified, payment_lock, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2338,7 +2486,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>payment_retry, inventory_reserved, amount_verified</t>
+          <t>payment_retry, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2360,7 +2508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>payment_processing, final_retry, inventory_reserved, amount_verified, payment_lock</t>
+          <t>payment_processing, final_retry, inventory_reserved, amount_verified, payment_lock, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2382,7 +2530,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>paid, payment_success, amount_verified, inventory_reserved</t>
+          <t>paid, payment_success, amount_verified, inventory_reserved, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2404,7 +2552,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>paid, payment_success, confirmation_retry, amount_verified</t>
+          <t>paid, payment_success, confirmation_retry, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2426,7 +2574,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>confirmed, paid, payment_success, amount_verified</t>
+          <t>confirmed, paid, payment_success, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2448,7 +2596,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>paid, payment_success, refund_pending, amount_verified</t>
+          <t>paid, payment_success, refund_pending, amount_verified, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2470,7 +2618,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>completed, paid, payment_success, amount_verified, terminal</t>
+          <t>completed, paid, payment_success, amount_verified, terminal, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2492,7 +2640,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cancelled, inventory_released, terminal</t>
+          <t>cancelled, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2514,7 +2662,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>failed, pre_payment_failure, inventory_unreserved, terminal</t>
+          <t>failed, pre_payment_failure, inventory_unreserved, terminal, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2536,7 +2684,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>failed, inventory_released, terminal</t>
+          <t>failed, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2558,7 +2706,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>refunded, payment_compensated, inventory_released, terminal</t>
+          <t>refunded, payment_compensated, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2578,7 +2726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="75" customWidth="1" min="1" max="1"/>
@@ -2594,70 +2742,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AG(!violation)</t>
+          <t>AG(no_invalid_transition)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AG(paid -&gt; payment_success)</t>
+          <t>AG(no_resource_conflict)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AG(completed -&gt; payment_success)</t>
+          <t>EF(payment_processing)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AG(cancelled -&gt; !payment_success)</t>
+          <t>EF(payment_success)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AG(failed -&gt; !payment_success)</t>
+          <t>EF(refund_pending)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AG(payment_pending -&gt; !payment_success)</t>
+          <t>EF(refunded)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AG(!resource_conflict)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>AG(refund_pending -&gt; payment_success)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>AG(refunded -&gt; payment_compensated)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AG(payment_processing -&gt; AF(terminal))</t>
+          <t>EF(terminal)</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2700,90 +2827,6 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>payment_success</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>cancelled</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>payment_success</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>payment_success</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>resource_conflict</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>payment_lock</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>resource_conflict</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>cancel_lock</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>two_success_payments</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>amount_mismatch</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>amount_verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>refunded</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>refund_pending</t>
         </is>
       </c>
     </row>
@@ -3054,19 +3097,25 @@
           <t>remaining_attempts, elapsed_ms</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>divide-by-zero</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1000</v>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3087,22 +3136,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>signature_code</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
+          <t>signature_code, callback_type</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>authentication-bypass</t>
+          <t/>
         </is>
       </c>
       <c r="G8" t="n">
         <v>4919</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sửa lỗi tồn kho âm khi đơn có sản phẩm trùng. Bổ sung validation Cart/User/Product và transaction giỏ hàng. Thêm migration bảo vệ tồn kho, giá và số lượng. Đồng bộ workbook, tạo bảng truy vết và manifest SHA-256.
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -1430,7 +1430,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28.8" customHeight="1">
+    <row r="26" ht="43.2" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
           <t>TC-25</t>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>5/5 PASS: xác thực/quyền sở hữu, rollback, idempotency, payment-cancel và concurrency được kiểm tra trên PostgreSQL</t>
+          <t>Tất cả test PASS, không SKIP; số lượng và verdict lấy từ application_tests.results.json. Kiểm tra quyền, idempotency, payment-cancel, validation và migration trên PostgreSQL</t>
         </is>
       </c>
       <c r="G26" s="1" t="inlineStr">
@@ -1541,7 +1541,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28.8" customHeight="1">
+    <row r="29" ht="43.2" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
           <t>TC-28</t>
@@ -1564,12 +1564,12 @@
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>Chạy pytest ATPM/atpm_project/python/tests/test_order_payment_spec.py và verify_teacher_spec.py</t>
+          <t>Chạy python security-analysis/verify_teacher_spec.py</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>Schema đúng 10 sheet; Excel/JSON đồng nghĩa; Kripke total và reachable; 7/7 CTL PASS; 6/6 test đặc tả PASS</t>
+          <t>Checker độc lập: schema đúng 10 sheet; Excel/JSON đồng nghĩa; Kripke total và reachable; 7/7 CTL PASS. Không thay thế lần chạy công cụ Windows của giảng viên.</t>
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">

</xml_diff>

<commit_message>
sua xlsx, pipelinejson va verificationjson
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1" style="1"/>
@@ -455,7 +455,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="57.6" customHeight="1">
+    <row r="3" ht="72.0" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>description</t>
@@ -463,7 +463,115 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Đặc tả kiểm chứng hình thức cho luồng Order-Payment: state machine có xử lý sự cố và phục hồi, safety/liveness, idempotency, serialization payment-cancel, bounded retry, compensation refund, SMT số học, fuzzing xác định, TLC, integration PostgreSQL và mô hình C về an toàn bộ nhớ.</t>
+          <t>Group 14 — Xây dựng và kiểm chứng an toàn hệ thống xử lý đơn hàng và thanh toán trực tuyến. Phạm vi đã làm: JWT/ownership/Admin, giá server, idempotency Order/Payment, consistency Order–Payment–Inventory, recovery charge/refund qua kill process và PostgreSQL stop/start, audit nguyên tử, admission, health/status, backup/restore, checkout/browser, model/SMT/fuzz và 5 module C minh họa an toàn bộ nhớ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18.0" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>updated_date</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 (Asia/Bangkok)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="43.2" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>evidence_baseline</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Evidence hiện lưu ngày 14/10/2026: 148/148 unit + 35/35 integration PASS, 0 SKIP (results/application_tests.results.json). Đây là kết quả đã lưu, không phải lần chạy mới khi cập nhật Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="43.2" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>coverage_baseline</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>InputValidator branch 97,22%; MoneyAmounts 100%; fuzz target branch 96,66%. Nguồn: security-analysis/results/coverage_summary.json và application_fuzzing.results.json; chỉ áp dụng target được đo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="57.6" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>model_scope</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>MoHinhTrangThai là recovery model trừu tượng 15 state, 37 event, 7 contract, không phải enum OrderStatus. PAYMENT_PROCESSING/PAYMENT_RETRY/PAYMENT_PROCESSING_FINAL kết hợp Order và Payment; CONFIRMATION_RETRY thuộc mở rộng thiết kế, chưa có scheduler/counter runtime. Xem IMPLEMENTATION_CONTRACTS.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43.2" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>liveness_scope</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>P10 progress-only lọc cạnh stutter; audit_liveness.py xác nhận raw AG AF terminal=false, progress-only=true. Đây không phải thuật toán fair-CTL đầy đủ; kết thúc còn phụ thuộc provider và hành động confirm/complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="43.2" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>generator_scope</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>HamSinhMa mô tả 5 module C BUGGY/FIXED học tập; không phải lỗi bộ nhớ của C# managed. KiemTraSoHoc là các bài toán số nguyên/cents, không phải phép toán Int32 trực tiếp trong production; app dùng decimal/guard, SMT dùng Z3 ngoài runtime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.6" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>verification_sources</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Nguồn trong security-analysis/: PHAM_VI_KIEM_CHUNG.md; IMPLEMENTATION_CONTRACTS.md; OPERATIONS.md; report/BAO_CAO.md; results/*.json và results/traceability_matrix.csv. Các tham chiếu rút gọn results/... trong workbook tính từ security-analysis/; lệnh chạy từ gốc repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="43.2" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>limitations</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Gateway là DurableFake local, chưa provider thu tiền thật. Chưa chứng minh mọi interleaving/crash window, partition, failover, power loss hoặc SLA production. Evidence/hash lúc đóng gói không tự chứng minh source của lần chạy lịch sử.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="43.2" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>future_work</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Ngoài nghiệm thu: tách DB migration/runtime role, retention job, webhook thật, shared Redis limiter, gateway thật, Kubernetes. Confirmation retry tự động còn là thiết kế; load chưa crossover/lặp để suy thống kê.</t>
         </is>
       </c>
     </row>
@@ -478,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1" style="1"/>
@@ -826,7 +934,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18.0" customHeight="1">
+    <row r="10" ht="43.2" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>TC-9</t>
@@ -834,27 +942,28 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>REQ-5, REQ-14</t>
+          <t>REQ-5, REQ-14, NFR-6</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Kiểm chứng mô hình Order kỳ vọng</t>
+          <t>Đối chiếu model Order ban đầu và model recovery</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>order_state_model.json hợp lệ</t>
+          <t>Có evidence model ban đầu và recovery model</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Chạy python security-analysis/run_analysis.py</t>
+          <t>Đọc results/order_state_model.results.json
+Chạy python3 security-analysis/verify_recovery_model.py và python3 security-analysis/audit_liveness.py</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>P1, P2, P3, P4 đều PASS</t>
+          <t>Model Order ban đầu có P1–P4 PASS trong phạm vi cũ; recovery 15 state là phạm vi mở rộng. Raw liveness recovery=false, progress-only=true theo policy lọc cạnh; không nhập nhằng hai model.</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
@@ -863,7 +972,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18.0" customHeight="1">
+    <row r="11" ht="43.2" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>TC-10</t>
@@ -881,17 +990,18 @@
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>order_state_model_buggy.json có cạnh lỗi</t>
+          <t>Model BUGGY có cạnh CANCELLED → PAID_AFTER_CANCELLED</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Chạy checker trên model BUGGY</t>
+          <t>Đọc results/order_state_model_buggy.results.json
+Chạy python3 security-analysis/verify_recovery_model.py để kiểm mutation tương ứng</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>P1 FAIL với CREATED → CANCELLED → PAID_AFTER_CANCELLED</t>
+          <t>P1 FAIL với witness CREATED → CANCELLED → PAID_AFTER_CANCELLED; mutation phải được phát hiện, đây là kết quả âm mong đợi.</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr">
@@ -977,7 +1087,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28.8" customHeight="1">
+    <row r="14" ht="43.2" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>TC-13</t>
@@ -985,27 +1095,28 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>REQ-4</t>
+          <t>REQ-4, NFR-2</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>Fuzz biên validator Order</t>
+          <t>Unit/coverage biên InputValidator</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>Có xUnit InputValidatorTests</t>
+          <t>InputValidatorTests và coverage evidence</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>Chạy các ca null/rỗng, amount, quantity, price, mismatch, nhiều item và giá trị biên</t>
+          <t>Kiểm null/rỗng, amount, quantity, price, mismatch, nhiều item và giá trị biên
+Đọc results/coverage_summary.json</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>Input sai bị từ chối; input ở biên hợp lệ được chấp nhận; branch coverage đạt ngưỡng</t>
+          <t>Snapshot 14/10/2026: InputValidator branch 97,22%, MoneyAmounts 100%; threshold 90% PASS. Đây là unit/coverage; random fuzz được ghi riêng tại TC-26.</t>
         </is>
       </c>
       <c r="G14" s="1" t="inlineStr">
@@ -1091,7 +1202,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="43.2" customHeight="1">
+    <row r="17" ht="57.6" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>TC-16</t>
@@ -1104,7 +1215,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>Kiểm chứng model phục hồi đầy đủ</t>
+          <t>Kiểm chứng recovery model hữu hạn</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -1114,13 +1225,13 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>Chạy python security-analysis/verify_recovery_model.py
-Đối chiếu 7 hợp đồng chức năng, 15 thuộc tính và tập state reachable</t>
+          <t>Chạy python3 security-analysis/verify_recovery_model.py
+Đọc results/order_payment_recovery_model.results.json</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>Model đúng có 7 hợp đồng, 15 state, 37 transition; P1-P15 PASS và tất cả state reachable</t>
+          <t>7 contract, 15 state, 37 event; P1–P15 PASS theo semantics của checker, mọi state reachable và 6/6 negative mutations được phát hiện. P10 chỉ progress-only; CONFIRMATION_RETRY thuộc thiết kế.</t>
         </is>
       </c>
       <c r="G17" s="1" t="inlineStr">
@@ -1281,7 +1392,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="28.8" customHeight="1">
+    <row r="22" ht="43.2" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
           <t>TC-21</t>
@@ -1289,28 +1400,28 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>REQ-16, REQ-17</t>
+          <t>REQ-16, REQ-17, REQ-19</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>Bounded retry và compensation</t>
+          <t>Retry hết budget vẫn giữ UNKNOWN an toàn</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>Model đúng, weak fairness được khai báo</t>
+          <t>PaymentServiceTests; provider trả UNKNOWN</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>Đi PAYMENT_PROCESSING → PAYMENT_RETRY → PAYMENT_PROCESSING_FINAL
-Thử timeout cuối và charged-but-commit-failed</t>
+          <t>Retry đến AttemptCount=2 rồi retry/reconcile tiếp; thử cancel
+Đọc source PaymentService và results/application_tests.results.json</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>Không có vòng retry tiến triển vô hạn; nhánh cuối tới FAILED hoặc REFUND_PENDING → REFUNDED</t>
+          <t>Không charge attempt thứ ba; UNKNOWN và reservation được giữ, cancel bị chặn; definitive result mới cho finalize. Confirmation retry tự động chưa hiện thực.</t>
         </is>
       </c>
       <c r="G22" s="1" t="inlineStr">
@@ -1467,7 +1578,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28.8" customHeight="1">
+    <row r="27" ht="57.6" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
           <t>TC-26</t>
@@ -1485,17 +1596,18 @@
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>Có corpus, seed cố định, timeout và crash policy</t>
+          <t>Corpus; seed=20261009; timeout=120s</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>Chạy python security-analysis/run_fuzzing.py</t>
+          <t>Chạy python3 security-analysis/run_fuzzing.py
+Đọc results/application_fuzzing.results.json và application-fuzzing-coverage.cobertura.xml</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>3/3 campaign PASS; 25.000 iteration cho validator và 25.000 transition; branch coverage 99,07%, không crash</t>
+          <t>Snapshot 14/10/2026: 3/3 campaign PASS, 25.000 iteration mỗi random campaign, branch target 96,66%, không crash/timeout. Target: InputValidator, PaymentValidator, OrderStateMachine, PaymentStateMachine, MoneyAmounts; không là coverage toàn app.</t>
         </is>
       </c>
       <c r="G27" s="1" t="inlineStr">
@@ -1504,7 +1616,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28.8" customHeight="1">
+    <row r="28" ht="57.6" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
           <t>TC-27</t>
@@ -1517,22 +1629,23 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>TLC kiểm chứng đặc tả TLA+</t>
+          <t>TLC kiểm chứng đặc tả TLA+ trong bound</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>Có tla2tools.jar</t>
+          <t>Có tla2tools.jar; đây là model TLA+ riêng</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>Chạy python security-analysis/run_tlc.py --jar /duong-dan/tla2tools.jar</t>
+          <t>Chạy python3 security-analysis/run_tlc.py --jar /duong-dan/tla2tools.jar
+Đọc results/tlc/OrderPayment.tlc.results.json</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>TLC không phát hiện lỗi: 35 state sinh, 20 state phân biệt, độ sâu 9; safety và liveness đều thỏa</t>
+          <t>Evidence TLC lịch sử: 35 state sinh, 20 phân biệt, độ sâu 9, không lỗi trong model/bound/assumptions đã khai báo. Không đổi nhãn thành lượt mới; không thay kết quả raw liveness của recovery graph hoặc proof runtime.</t>
         </is>
       </c>
       <c r="G28" s="1" t="inlineStr">
@@ -1573,6 +1686,840 @@
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="43.2" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>TC-29</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>REQ-14, CON-8, NFR-6</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>Audit riêng semantics liveness</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>Recovery graph đầy đủ có cạnh stutter</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/audit_liveness.py
+Đọc results/liveness_audit.results.json và counterexample_lasso</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>Raw AG AF terminal=false và có lasso; progress-only=true sau lọc cạnh. Verdict audit PASS là phát hiện đúng khác biệt này, không là proof fair-CTL hoặc runtime luôn kết thúc.</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="43.2" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>REQ-17, REQ-20</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Kill API sau charge journal, trước finalize</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>ProcessRestartTests; PostgreSQL/ledger tạm</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Kill OS process tại marker sau journal publish; khởi động process mới cùng DB/ledger
+Đọc results/process_restart.results.json</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>Worker mới tự phục hồi SUCCESS/PAID, một payment/journal charge, AttemptCount=1, journal không đổi và kho vẫn reserved. Chỉ bao phủ crash window đã chọn.</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="43.2" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>REQ-17, REQ-20, CON-9</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Kill API sau refund journal, trước finalize</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>RefundRestartTests; charge thành công, refund pending</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>Kill process sau refund publish; restart cùng DB/ledger và đợi worker
+Đọc results/refund_restart.results.json</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>REFUNDED, charge reference giữ nguyên, journal refund không đổi, PendingSince xóa và stock release đúng một lần; replay không tạo refund mới.</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="57.6" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>TC-32</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>REQ-19, REQ-20, REQ-25</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>Charge recovery sau PostgreSQL stop/start</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>PostgresReconnectTests; local PostgreSQL binaries; DurableFake</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/run_recovery_demo.py
+Đọc results/postgres_reconnect_charge.results.json</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>Cùng API process/pool, ready 200→503→200, live=200 khi DB tắt; finalize=503, worker scan failure rồi recovery. Charge=1, payment=1, AttemptCount=1, SUCCESS/PAID/RESERVED; reserve=1, release=0, stock 50→49, journal giữ hash.</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="57.6" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>TC-33</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>REQ-17, REQ-20, REQ-25</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Refund recovery sau PostgreSQL stop/start</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>PostgresReconnectTests; charge thành công; local PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/run_recovery_demo.py
+Đọc results/postgres_reconnect_refund.results.json</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>Cùng API process/pool, ready 200→503→200; charge=1/refund=1, giữ charge reference và key/hash journal. Payment/Order REFUNDED, inventory RELEASED, release=1, stock trở về 50; replay không release lại.</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="57.6" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>TC-34</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>REQ-19, NFR-7</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Timeout gateway và late result</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>GatewayTimeoutTests với adapter không hợp tác cancellation</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Kiểm charge/refund/charge-status/refund-status, late success, worker progress và shutdown
+Đọc results/application_tests.results.json</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>Caller waiting có bound; timeout charge giữ UNKNOWN/reservation, timeout refund giữ REFUND_PENDING; late result không tự finalize. Worker tiếp tục candidate khác và shutdown không invent outcome.</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="57.6" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>TC-35</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>REQ-21, CON-10</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>Replay receipt qua hai host và bind payload/customer</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>AtomicAuditIdempotencyTests, hai host dùng chung PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Tạo Order có key, replay qua host khác sau cancel/catalog đổi; đổi payload hoặc JWT customer; thử key sai/đa trị</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Cùng customer/key/payload trả 201, cùng ID/Location/original receipt; payload đổi trả 409, customer khác có namespace riêng. Key sai trả 400; đọc trạng thái mới qua GET, không dùng receipt cũ làm live state.</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="43.2" customHeight="1">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>TC-36</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>REQ-3, REQ-18, REQ-21, CON-11</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Concurrent same-key và không oversell</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>AtomicAuditIdempotencyTests; PostgreSQL thật</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Gửi same-key đồng thời; retry cùng payload/key sau conflict
+Cho hai host tranh 10 đơn vị tồn kho; kiểm duplicate ProductId lines</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>Chỉ một reserve/Order cho cùng key; tổng stock được bảo toàn, không âm hoặc oversell. Conflict có thể trả 409; duplicate lines phải được cộng dồn trước stock guard.</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="57.6" customHeight="1">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>TC-37</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>REQ-22, NFR-1, NFR-8</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>COMMIT audit nguyên tử và direct SQL rollback</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>AtomicAuditIdempotencyTests; DB audit triggers</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Làm audit INSERT thất bại khi tạo Order; kiểm stock/Order rollback
+Thử direct SQL mutation rồi rollback/commit</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>Audit COMMIT lỗi rollback cả nghiệp vụ; rollback nghiệp vụ bỏ audit tương ứng; commit lưu audit resource ID thật. Request metadata không bị lẫn qua pooled connections, SQL không có request actor ghi SYSTEM.</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57.6" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>TC-38</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>REQ-22, NFR-3, NFR-8</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>BEGIN/RESULT fail và audit append-only</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>AdmissionAuditTests/AuditMiddlewareTests</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Gây lỗi BEGIN, lỗi RESULT sau commit; kiểm correlation/redaction
+Thử UPDATE/DELETE/TRUNCATE AuditEvents</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>BEGIN lỗi: 503 trước business action; RESULT lỗi: 503 requiresReconciliation=true dù business có thể đã commit. Trigger chặn sửa/xóa audit; không có password/JWT/raw key/body. DBA vẫn nằm ngoài bảo đảm append-only.</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="43.2" customHeight="1">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>TC-39</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>REQ-23</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>Rate/body/item admission boundaries</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>AdmissionAuditTests, BodyLimitTests, AdmissionBoundaryTests</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>Kiểm auth/API bucket riêng, verified-user buckets, 429/Retry-After
+Thử body có/không Content-Length, streaming quá cap và vượt item count</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>Quota vượt trả 429 không queue; body vượt trả 413 trước JSON binding, item vượt bị từ chối trước persistence. 429/413 trước audit không ghi BEGIN/RESULT; limiter chỉ local mỗi process.</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72.0" customHeight="1">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>TC-40</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>REQ-24, CON-13</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>Checkout retry/key/payload qua mocked browser</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>Chrome/Chromium; browser/checkout_retry.template.html; OrderRetryContractTests</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/verify_checkout.py
+Kiểm metadata 409, wrapped SQLSTATE, stable body/key, jitter, abort và double submit</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>Tối đa 4 attempts/8s; chỉ ORDER_CONCURRENT_WRITE + retryable=true mới auto retry với backoff. 503/network/401/403/429 hoặc hết budget giữ key; không retry generic DB/business errors. Evidence: results/checkout_retry.results.json; mocked fetch không là live API.</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="57.6" customHeight="1">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>TC-41</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>REQ-25</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>Health, quyền operations và pending age</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>OperationsTests; PendingAgeTests</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Gọi /health/live, /health/ready, /api/operations/status với anonymous/user/Admin
+Reconcile UNKNOWN nhiều lần, tiến clock quan sát và gây audit append failure</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>Health tối thiểu, status chỉ Admin/no-store/redacted; UpdatedAt refresh không reset PendingSince, stuck vẫn được phát hiện; audit failure có counter/alert. Clock thử chỉ phục vụ quan sát, không thay outcome provider.</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="57.6" customHeight="1">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>TC-42</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>REQ-26</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>Backup/restore DB cùng gateway ledger</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>OperationalDrillTests; local PostgreSQL; tài nguyên tạm</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Restore snapshot sang cluster riêng rồi khởi động API/worker
+Đọc results/backup_restore.results.json</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>Snapshot đã lưu PASS: hash dữ liệu 9 bảng khớp, 4 audit triggers hoạt động, sequence cấp ID mới, receipt replay được, pending charge recovered với charge=1/AttemptCount=1; DB nguồn không đổi. Timing không là SLA/RPO/RTO.</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="57.6" customHeight="1">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>TC-43</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>REQ-24, NFR-10</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>Đo bounded retry qua hai API process</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>OrderRetryLoadTests; 8 users, 4 products, concurrency=8</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>So sánh one-shot và retry policy: 96 logical requests/scenario
+Đọc raw samples/backoff trong results/order_retry_load.results.json</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>PASS các invariant bounded attempts, no duplicate, conservation stock, COMMIT count; driver C# mô phỏng policy, JS được kiểm riêng. Baseline chạy trước, chưa crossover/repetitions/statistical confidence; không suy SLA.</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="43.2" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>TC-44</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>REQ-27</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Live browser với normal application và PostgreSQL thật</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>ApplicationSmokeTests; Chrome CDP; PostgreSQL/ledger tạm</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Chạy NormalApplicationServesShopAndCompletesRealBrowserFlow
+Đọc results/application_smoke.results.json</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Register/login→cart→order→fake payment→history PASS; reload/session và logout đúng; double submit được kiểm, không gửi card fields. Đây là HTTP/DB thật, khác browser mocked-fetch retry.</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="57.6" customHeight="1">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>TC-45</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>REQ-4, CON-2, CON-11</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>Fractional cents và DB CHECK</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>MoneyPrecisionTests; PostgreSQL HTTP regression</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>Gửi 25,001/25,005 và cent hợp lệ 25,01/25,0100; thử raw SQL Stock âm/Quantity không dương
+Đọc results/application_tests.results.json</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>Fractional cent bị từ chối trước persistence; cent hợp lệ round-trip, trailing zeroes được nhận. DB CHECK chặn Stock&lt;0/Quantity≤0; bound Quantity≤10000 do app kiểm. Không suy cents guard application ngăn raw SQL tự round numeric.</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="43.2" customHeight="1">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>TC-46</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>REQ-17, NFR-6</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>Mutation paid thất bại không compensation</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>BUG-PAID-FAILED-WITHOUT-REFUND trong recovery checker</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/verify_recovery_model.py
+Đọc negative_scenarios trong results/order_payment_recovery_model.results.json</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>Phát hiện mutation chuyển paid sang FAILED bỏ refund; trả counterexample/property failure. Không dùng kết quả này để khẳng định tự động confirmation retry đã có trong source.</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="43.2" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>TC-47</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>REQ-19, NFR-6</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>Mutation UNKNOWN trả kho sớm</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>BUG-UNKNOWN-RELEASED trong recovery checker</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/verify_recovery_model.py
+Đọc negative_scenarios trong results/order_payment_recovery_model.results.json</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>Phát hiện UNKNOWN bị terminal hóa hoặc release reservation trước definitive outcome; có counterexample vi phạm policy UNKNOWN an toàn.</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="43.2" customHeight="1">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>TC-48</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>NFR-9</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>Đối chiếu snapshot nghiệm thu toàn suite</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>results/application_tests.results.json; không thay summary bằng filtered tests</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Đọc suites.unit/suites.integration và thời điểm TRX; đối chiếu report/BAO_CAO.md
+Khi chạy lại dùng lệnh toàn suite trong README.md</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Snapshot 14/10/2026: unit 148/148, integration 35/35 PASS, fail=0, skip=0. Lần cập nhật workbook không là lần chạy lại .NET; source/hash và giới hạn lịch sử được ghi riêng.</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="43.2" customHeight="1">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>TC-49</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>NFR-10, REQ-23</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Load probe latency/conflict/throttle</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>OperationalDrillTests; hai real API process</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>Đọc raw samples/status counts/nearest-rank p95/p99 trong results/load_probe.results.json</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>Load probe đã lưu PASS các oracle stock và admission; hot-product one-shot có thể 409. Successful/s và latency chỉ là quan sát workload; quota local không thành shared quota.</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="57.6" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>TC-50</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>REQ-3, CON-11</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>SMT tổng quantity của các dòng cùng sản phẩm</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>Z3; Security/InventoryVerification.z3</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>Chạy python3 security-analysis/verify_inventory_smt.py
+Đọc results/inventory_verification.results.json</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>3/3 ca SAT/UNSAT đúng kỳ vọng: baseline stock=10, q1=q2=6 có oversell; aggregated guard không cho stock âm, nhận đúng stock. Model hai dòng một sản phẩm với số nguyên toán học, không chứng minh EF/interleaving/API đầy đủ.</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1589,7 +2536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1" style="1"/>
@@ -1664,7 +2611,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28.8" customHeight="1">
+    <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>REQ-3</t>
@@ -1672,7 +2619,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Khi tạo đơn, giá sản phẩm phải lấy từ cơ sở dữ liệu phía server, sản phẩm phải tồn tại/đang hoạt động và tồn kho phải đủ.</t>
+          <t>Tạo Order lấy UnitPrice/TotalAmount từ catalog server; kiểm sản phẩm tồn tại/active và cộng dồn quantity theo ProductId trước kiểm stock. Payload giá/tổng không hợp lệ bị từ chối; client UnitPrice không là nguồn giá có thẩm quyền.</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -1686,7 +2633,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28.8" customHeight="1">
+    <row r="5" ht="57.6" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>REQ-4</t>
@@ -1694,7 +2641,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>TotalAmount phải dương, trong giới hạn cho phép và khớp tổng Quantity × UnitPrice với sai số tối đa 0,01; dữ liệu sai phải bị từ chối.</t>
+          <t>Price/TotalAmount/Payment.Amount phải là bội 0,01 trong giới hạn; fractional cent bị từ chối, không round âm thầm. InputValidator/OrderService chấp nhận lệch tổng tối đa 0,01; Order lưu tổng giá server, Payment phải bằng chính xác tổng đã lưu.</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -1708,7 +2655,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="43.2" customHeight="1">
+    <row r="6" ht="57.6" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>REQ-5</t>
@@ -1716,7 +2663,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Order chỉ được chuyển theo chuỗi CREATED → VALIDATED → PAYMENT_PENDING → PAID → CONFIRMED → COMPLETED; không bỏ bước, quay ngược hoặc hồi sinh trạng thái terminal.</t>
+          <t>Order đi CREATED → VALIDATED → PAYMENT_PENDING → PAID → CONFIRMED → COMPLETED; cho phép cancel trước charge, FAILED khi decline, PAID/CONFIRMED → REFUND_PENDING → REFUNDED. Guard cấm hồi sinh terminal; model có các state trừu tượng bổ sung, không đồng nhất với enum runtime.</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -1906,7 +2853,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28.8" customHeight="1">
+    <row r="15" ht="43.2" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>REQ-14</t>
@@ -1914,7 +2861,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Từ mọi trạng thái Order có thể đạt tới, mọi đường thực thi hữu hạn tiến triển phải cuối cùng tới COMPLETED, CANCELLED hoặc FAILED.</t>
+          <t>Liveness có điều kiện: checker progress-only đạt terminal khi lọc các cạnh đánh dấu stutter. Raw AG AF terminal trên graph đầy đủ là false; không suy ra runtime luôn kết thúc khi provider còn UNKNOWN.</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
@@ -1950,7 +2897,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28.8" customHeight="1">
+    <row r="17" ht="57.6" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>REQ-16</t>
@@ -1958,12 +2905,12 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Retry thanh toán và xác nhận phải có bound; khi hết ngân sách retry phải chuyển FAILED hoặc REFUND_PENDING thay vì lặp vô hạn.</t>
+          <t>PaymentService giới hạn charge tối đa 2 attempts cho cùng logical payment/key. Hết budget mà UNKNOWN vẫn giữ reservation và chỉ lookup/reconcile; không suy thành FAILED. Bounded confirmation retry chỉ có trong model, chưa hiện thực scheduler/counter tự động.</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>liveness</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -1972,7 +2919,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="43.2" customHeight="1">
+    <row r="18" ht="57.6" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>REQ-17</t>
@@ -1980,7 +2927,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Nếu gateway đã charge nhưng không thể hoàn tất đơn hoặc commit PAID, hệ thống phải dùng REFUND_PENDING và REFUNDED để bù trừ; không được đổi thẳng sang FAILED.</t>
+          <t>Charge đã xảy ra nhưng finalize PAID lỗi phải được lookup bằng cùng key và hoàn tất SUCCESS/PAID, không charge mù hoặc đổi FAILED. Khi yêu cầu refund cho Order PAID/CONFIRMED, dùng REFUND_PENDING → REFUNDED, giữ dấu vết charge và release kho một lần.</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -2013,6 +2960,204 @@
       <c r="D19" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="43.2" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>REQ-19</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSING/UNKNOWN phải được worker reconciliation hỏi trạng thái charge cũ; REFUND_PENDING hỏi trạng thái refund cũ. Lookup không tăng AttemptCount, không tự phát charge/refund; UNKNOWN giữ reservation và chặn cancel.</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.6" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>REQ-20</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Với DurableFake journal đã publish trước local finalize, API kill/restart hoặc PostgreSQL stop/start phải phục hồi đúng charge/refund. Reconnect giữ nguyên API process/pool; giữ key, transaction reference và journal, không duplicate operation hoặc release kho.</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="57.6" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>REQ-21</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>POST /api/orders hỗ trợ Idempotency-Key tùy chọn, namespace theo customer từ JWT. Cùng key/payload trả 201 và receipt gốc kể cả sau cancel/catalog đổi; payload khác trả 409. Unique key hash, reserve, order và receipt commit cùng transaction; client không key vẫn có thể tạo Order mới.</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="57.6" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>REQ-22</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Mutation Orders/Payments phải có COMMIT audit cùng transaction bằng DB trigger; audit lỗi phải rollback nghiệp vụ. BEGIN/RESULT HTTP dùng correlation server và allowlist không có secrets; BEGIN lỗi trả 503 trước action, RESULT lỗi sau action trả 503 với requiresReconciliation=true.</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.6" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>REQ-23</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Admission mặc định body ≤65536 byte, tối đa 100 order items, auth 10 request/60s theo connection IP, API 120 request/60s theo subject hoặc IP. Quá quota trả 429/Retry-After; body quá lớn trả 413 cả khi thiếu Content-Length, trước JSON binding.</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.6" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>REQ-24</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Checkout giữ attempt/key/payload theo tài khoản trong sessionStorage; chặn double submit và thay payload khi outcome chưa rõ. Create-order retry tối đa 4 HTTP attempts/8s, chỉ cho 409 ORDER_CONCURRENT_WRITE với retryable=true; 503/network giữ key để đối soát.</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.6" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>REQ-25</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Health live/ready trả thông tin tối thiểu; ready phản ánh DB outage. /api/operations/status chỉ Admin, no-store và không lộ secret; PendingSince giữ tuổi unresolved qua status lookup, có chỉ số recovery/audit failure và cảnh báo pending quá lâu.</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57.6" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>REQ-26</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Backup/restore trên môi trường tạm phải giữ database, receipt, audit triggers, identity sequence và gateway ledger nhất quán; worker phục hồi pending charge sau restore không charge lại. Không dùng phép đo drill làm cam kết RPO/RTO.</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="43.2" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>REQ-27</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Shop chạy được register/login → cart → order → payment giả lập → history qua HTTP/PostgreSQL thật; reload/logout đúng, không thu/gửi card fields. Browser smoke và browser mocked-fetch có phạm vi bằng chứng riêng.</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -2027,7 +3172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1" style="1"/>
@@ -2052,7 +3197,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28.8" customHeight="1">
+    <row r="2" ht="57.6" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NFR-1</t>
@@ -2060,7 +3205,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Các thay đổi Order, tồn kho và Payment phải được lưu nguyên tử; luồng dùng PostgreSQL phải chạy trong transaction mức Serializable.</t>
+          <t>Các mutation aggregate Order–Payment–Inventory dùng transaction Serializable trên PostgreSQL. Lưu PROCESSING/REFUND_PENDING trước khi gọi gateway; finalize là transaction riêng. Gateway và DB không có distributed transaction, khoảng hở được reconciliation xử lý.</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -2069,7 +3214,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28.8" customHeight="1">
+    <row r="3" ht="43.2" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>NFR-2</t>
@@ -2077,7 +3222,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Branch coverage của lớp kiểm tra đầu vào và các guard trạng thái trọng yếu phải đạt tối thiểu 90% trong pipeline kiểm thử.</t>
+          <t>Branch coverage tối thiểu 90% cho target đã đo: InputValidator và tập target fuzz được chọn. Coverage không đại diện toàn ứng dụng; ghi số đo và thời điểm từ coverage_summary.json/application_fuzzing.results.json.</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -2151,6 +3296,74 @@
       <c r="C7" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43.2" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>NFR-7</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Timeout wrapper charge/refund/status mặc định 5000ms, startup validate 50..60000ms. Caller không chờ vô hạn; late result không tự ghi state. Adapter không hợp tác chưa có cơ chế cưỡng chế dừng, backpressure vẫn là giới hạn.</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="43.2" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>NFR-8</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>AuditEvents append-only chặn UPDATE/DELETE/TRUNCATE bằng PostgreSQL trigger; COMMIT audit chỉ bảo vệ Orders/Payments. Không chống DBA đổi schema/disable trigger; chưa có retention job hoặc chữ ký chống sửa log.</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="43.2" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>NFR-9</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả nghiệm thu phải ghi total/pass/fail/skip, thời điểm, source/artifact hash khi có và giới hạn. Demo filtered tests không ghi đè summary toàn suite; snapshot evidence không là lần chạy mới.</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="43.2" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>NFR-10</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Load/race phải kiểm no duplicate, conservation stock, bounded attempts và COMMIT count. Báo raw samples/p95/p99/status; workload hai API process hữu hạn và limiter local không chứng minh shared quota hoặc SLA production.</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -2165,7 +3378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1" style="1"/>
@@ -2190,7 +3403,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28.8" customHeight="1">
+    <row r="2" ht="43.2" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>CON-1</t>
@@ -2198,7 +3411,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Ứng dụng dùng ASP.NET Core/.NET 10, Entity Framework Core và PostgreSQL; API trao đổi JSON qua REST.</t>
+          <t>Ứng dụng dùng ASP.NET Core/.NET 10, Entity Framework Core và PostgreSQL; REST JSON. Các module hiện chạy chung một host và một database, chưa triển khai thành các microservice độc lập.</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -2241,7 +3454,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28.8" customHeight="1">
+    <row r="5" ht="57.6" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>CON-4</t>
@@ -2249,7 +3462,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Order terminal gồm COMPLETED, CANCELLED và FAILED; mô hình Kripke dùng self-loop ở trạng thái terminal để quan hệ chuyển là total.</t>
+          <t>Order terminal trong source gồm COMPLETED, CANCELLED, FAILED, REFUNDED. PRE_PAYMENT_REJECTED là trạng thái trừu tượng của model, không lưu Order khi tạo thất bại. Self-loop terminal trong Kripke biểu diễn no-op/reject, không là mutation được source cho phép.</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -2292,7 +3505,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28.8" customHeight="1">
+    <row r="8" ht="43.2" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t>CON-7</t>
@@ -2300,7 +3513,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Model dùng tối đa một lần retry thanh toán cuối; PAYMENT_PROCESSING_FINAL không được quay lại PAYMENT_RETRY.</t>
+          <t>Runtime MaxChargeAttempts=2. Model PAYMENT_PROCESSING_FINAL vẫn có cạnh final_payment_unknown/final_charged_but_commit_failed → PAYMENT_RETRY để giữ UNKNOWN; graph không mã hóa đầy đủ counter runtime và không là proof bound mọi đường thực thi.</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -2309,7 +3522,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28.8" customHeight="1">
+    <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>CON-8</t>
@@ -2317,7 +3530,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Thuộc tính liveness dùng weak fairness: cạnh no-op/retry được đánh dấu stutter có thể lặp, nhưng transition tiến triển đang enable cuối cùng phải chạy.</t>
+          <t>Weak fairness là assumption được khai báo trong model. Checker hiện bỏ cạnh metadata stutter để kiểm progress-only, kể cả vài cạnh đổi state; raw AG AF terminal=false. Không diễn giải PASS thành fair-CTL hoặc bảo đảm provider cuối cùng trả kết quả.</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -2326,7 +3539,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="28.8" customHeight="1">
+    <row r="10" ht="43.2" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>CON-9</t>
@@ -2334,12 +3547,97 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Refund dùng idempotency key riêng; callback refund trùng chỉ trả kết quả đã lưu và không hoàn tiền lần hai.</t>
+          <t>Refund có idempotency key riêng, bind charge transaction reference; replay/lookup không refund lần hai. Gateway callback được xác thực chỉ là assumption của model, chưa có webhook adapter thật.</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="43.2" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>CON-10</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Order Idempotency-Key: một header value, 1..128 ký tự visible ASCII; DB lưu SHA-256 key/payload và original receipt, unique(CustomerId, CreationKeyHash). Khác Payment.IdempotencyKey trong JSON; không suy hai namespace là một.</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.6" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>CON-11</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>PostgreSQL CHECK chặn Stock âm và Quantity không dương; bound Quantity≤10000 thuộc application guard. Concurrency token/unique index/Serializable hỗ trợ chống stale write và oversell. Application cents guard không ngăn raw SQL tự round numeric(18,2).</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43.2" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>CON-12</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>DurableFake mặc định là journal local ngoài wwwroot, file name SHA-256 và publish temp/flush/rename; chỉ mô phỏng provider bền qua process restart. MemoryFake dùng cho một số fixture, không có độ bền qua restart.</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="43.2" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>CON-13</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Runtime retry create order chỉ allowlist DbUpdateConcurrencyException, 40001/40P01 hoặc 23505 đúng index creation key; retryable=true cần key hợp lệ. Generic 23505/23514, business conflict và audit failure không tự retry.</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="43.2" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>CON-14</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Local PostgreSQL stop/start, OS process kill, backup/restore và browser được kiểm trên tài nguyên test tạm. DB RBAC tách role, retention, webhook/gateway thật, distributed limiter và Kubernetes nằm ngoài nghiệm thu.</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -2841,7 +4139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3074,86 +4372,6 @@
       </c>
       <c r="H6" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>safe_divide_retry_budget</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>divide</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>remaining_attempts, elapsed_ms</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>verify_gateway_callback</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>magic_value</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>signature_code, callback_type</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>4919</v>
-      </c>
-      <c r="H8" t="n">
-        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dong bo so lieu 149 test, bo sung tai lieu nghiem thu va don TODO sai
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15 (Asia/Bangkok)</t>
+          <t>2026-10-22 (Asia/Bangkok)</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Evidence hiện lưu ngày 14/10/2026: 148/148 unit + 35/35 integration PASS, 0 SKIP (results/application_tests.results.json). Đây là kết quả đã lưu, không phải lần chạy mới khi cập nhật Excel.</t>
+          <t>Evidence hiện lưu ngày 22/10/2026: 149/149 unit + 35/35 integration PASS, 0 SKIP (results/application_tests.results.json). Số liệu lấy từ lần chạy toàn suite gần nhất; đọc trực tiếp suites.unit/suites.integration thay vì chép tay.</t>
         </is>
       </c>
     </row>
@@ -499,7 +499,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>InputValidator branch 97,22%; MoneyAmounts 100%; fuzz target branch 96,66%. Nguồn: security-analysis/results/coverage_summary.json và application_fuzzing.results.json; chỉ áp dụng target được đo.</t>
+          <t>InputValidator branch 97,22%; MoneyAmounts 100%; fuzz target branch 97,50%. Nguồn: security-analysis/results/coverage_summary.json và application_fuzzing.results.json; chỉ áp dụng target được đo.</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="57.6" customHeight="1">
+    <row r="27" ht="86.4" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
           <t>TC-26</t>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>Snapshot 14/10/2026: 3/3 campaign PASS, 25.000 iteration mỗi random campaign, branch target 96,66%, không crash/timeout. Target: InputValidator, PaymentValidator, OrderStateMachine, PaymentStateMachine, MoneyAmounts; không là coverage toàn app.</t>
+          <t>4 campaign: corpus, validator random, state-pair random và stateful aggregate (2.000 sequence × tối đa 20 step). Random campaign dùng 25.000 iteration; stateful kiểm Order–Payment–Inventory invariant sau mỗi thao tác. Coverage chỉ áp dụng target được đo, không là coverage toàn app hoặc fuzz HTTP/concurrency/gateway thật.</t>
         </is>
       </c>
       <c r="G27" s="1" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>Snapshot 14/10/2026: unit 148/148, integration 35/35 PASS, fail=0, skip=0. Lần cập nhật workbook không là lần chạy lại .NET; source/hash và giới hạn lịch sử được ghi riêng.</t>
+          <t>Snapshot 22/10/2026: unit 149/149, integration 35/35 PASS, fail=0, skip=0. Số liệu lấy từ TRX của lần chạy toàn suite gần nhất; source/hash và giới hạn lịch sử được ghi riêng.</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">

</xml_diff>

<commit_message>
nang workbook ATPM dat checklist P1 va dong bo recovery model 14 state
</commit_message>
<xml_diff>
--- a/OrderPaymentMicroservice_Security_Spec.xlsx
+++ b/OrderPaymentMicroservice_Security_Spec.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1" style="1"/>
@@ -511,65 +511,77 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>MoHinhTrangThai là recovery model trừu tượng 15 state, 37 event, 7 contract, không phải enum OrderStatus. PAYMENT_PROCESSING/PAYMENT_RETRY/PAYMENT_PROCESSING_FINAL kết hợp Order và Payment; CONFIRMATION_RETRY thuộc mở rộng thiết kế, chưa có scheduler/counter runtime. Xem IMPLEMENTATION_CONTRACTS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="43.2" customHeight="1">
+          <t>MoHinhTrangThai là recovery model trừu tượng 14 state, 35 event, 7 contract, không phải enum OrderStatus. PAYMENT_PROCESSING/PAYMENT_RETRY/PAYMENT_PROCESSING_FINAL kết hợp Order và Payment; không còn state confirmation-retry vì runtime không có scheduler/counter tương ứng. Workbook thêm cụm khóa minh họa theo ATPM §3.5. Xem IMPLEMENTATION_CONTRACTS.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72.0" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>liveness_scope</t>
+          <t>lock_cluster_scope</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>P10 progress-only lọc cạnh stutter; audit_liveness.py xác nhận raw AG AF terminal=false, progress-only=true. Đây không phải thuật toán fair-CTL đầy đủ; kết thúc còn phụ thuộc provider và hành động confirm/complete.</t>
+          <t>Cụm free/main_holds/log_holds/conflict được thêm đúng checklist ATPM §3.5–3.7. Nhãn safe/main_locked/log_locked/violation và cạnh main_holds→conflict là bài tập phát hiện lỗi: pipeline sẽ báo CWE-667/CWE-693 tại conflict. Đây là hành vi đúng thiết kế của đề bài, không phải lỗi runtime của OrderPaymentMicroservice; 14 state nghiệp vụ vẫn được kiểm bởi recovery checker.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="43.2" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>generator_scope</t>
+          <t>liveness_scope</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>HamSinhMa mô tả 5 module C BUGGY/FIXED học tập; không phải lỗi bộ nhớ của C# managed. KiemTraSoHoc là các bài toán số nguyên/cents, không phải phép toán Int32 trực tiếp trong production; app dùng decimal/guard, SMT dùng Z3 ngoài runtime.</t>
+          <t>P10 progress-only lọc cạnh stutter; audit_liveness.py xác nhận raw AG AF terminal=false, progress-only=true. Đây không phải thuật toán fair-CTL đầy đủ; kết thúc còn phụ thuộc provider và hành động confirm/complete.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="57.6" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
+          <t>generator_scope</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>HamSinhMa mô tả 5 module C BUGGY/FIXED và 2 hàm Python (divide/magic_value) học tập; không phải lỗi bộ nhớ của C# managed. KiemTraSoHoc là các bài toán cộng dồn số nguyên/cents theo ngưỡng int16/uint16/int32/uint32 của ATPM, không phải phép toán Int32 trực tiếp trong production; app dùng decimal/guard, SMT dùng Z3 ngoài runtime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="57.6" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
           <t>verification_sources</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Nguồn trong security-analysis/: PHAM_VI_KIEM_CHUNG.md; IMPLEMENTATION_CONTRACTS.md; OPERATIONS.md; report/BAO_CAO.md; results/*.json và results/traceability_matrix.csv. Các tham chiếu rút gọn results/... trong workbook tính từ security-analysis/; lệnh chạy từ gốc repository.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="43.2" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>limitations</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Gateway là DurableFake local, chưa provider thu tiền thật. Chưa chứng minh mọi interleaving/crash window, partition, failover, power loss hoặc SLA production. Evidence/hash lúc đóng gói không tự chứng minh source của lần chạy lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="43.2" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
+          <t>limitations</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Gateway là DurableFake local, chưa provider thu tiền thật. Chưa chứng minh mọi interleaving/crash window, partition, failover, power loss hoặc SLA production. Evidence/hash lúc đóng gói không tự chứng minh source của lần chạy lịch sử.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43.2" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
           <t>future_work</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Ngoài nghiệm thu: tách DB migration/runtime role, retention job, webhook thật, shared Redis limiter, gateway thật, Kubernetes. Confirmation retry tự động còn là thiết kế; load chưa crossover/lặp để suy thống kê.</t>
         </is>
@@ -963,7 +975,7 @@
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>Model Order ban đầu có P1–P4 PASS trong phạm vi cũ; recovery 15 state là phạm vi mở rộng. Raw liveness recovery=false, progress-only=true theo policy lọc cạnh; không nhập nhằng hai model.</t>
+          <t>Model Order ban đầu có P1–P4 PASS trong phạm vi cũ; recovery 14 state là phạm vi mở rộng. Raw liveness recovery=false, progress-only=true theo policy lọc cạnh; không nhập nhằng hai model.</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
@@ -1231,7 +1243,7 @@
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>7 contract, 15 state, 37 event; P1–P15 PASS theo semantics của checker, mọi state reachable và 6/6 negative mutations được phát hiện. P10 chỉ progress-only; CONFIRMATION_RETRY thuộc thiết kế.</t>
+          <t>7 contract, 14 state, 35 event; P1–P15 PASS theo semantics của checker, mọi state reachable và 6/6 negative mutations được phát hiện. P10 chỉ progress-only; không còn state confirmation-retry không có runtime.</t>
         </is>
       </c>
       <c r="G17" s="1" t="inlineStr">
@@ -1421,7 +1433,7 @@
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>Không charge attempt thứ ba; UNKNOWN và reservation được giữ, cancel bị chặn; definitive result mới cho finalize. Confirmation retry tự động chưa hiện thực.</t>
+          <t>Không charge attempt thứ ba; UNKNOWN và reservation được giữ, cancel bị chặn; definitive result mới cho finalize. Confirmation failure giữ PAID để Admin confirm/refund, không tự charge lại.</t>
         </is>
       </c>
       <c r="G22" s="1" t="inlineStr">
@@ -1654,7 +1666,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="43.2" customHeight="1">
+    <row r="29" ht="72.0" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
           <t>TC-28</t>
@@ -1682,7 +1694,7 @@
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>Checker độc lập: schema đúng 10 sheet; Excel/JSON đồng nghĩa; Kripke total và reachable; 7/7 CTL PASS. Không thay thế lần chạy công cụ Windows của giảng viên.</t>
+          <t>Checker độc lập: schema đúng 10 sheet; Excel/JSON đồng nghĩa; Kripke total và reachable; 10 CTL (9 đúng, AG(!violation) false có chủ đích); 6 cặp mutex, dòng đầu bị conflict vi phạm có chủ đích → CWE-667/693. Không thay lần chạy công cụ Windows của giảng viên.</t>
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">
@@ -2905,7 +2917,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>PaymentService giới hạn charge tối đa 2 attempts cho cùng logical payment/key. Hết budget mà UNKNOWN vẫn giữ reservation và chỉ lookup/reconcile; không suy thành FAILED. Bounded confirmation retry chỉ có trong model, chưa hiện thực scheduler/counter tự động.</t>
+          <t>PaymentService giới hạn charge tối đa 2 attempts cho cùng logical payment/key. Hết budget mà UNKNOWN vẫn giữ reservation và chỉ lookup/reconcile; không suy thành FAILED. Không có automatic confirmation retry trong source; Admin confirm hoặc refund thủ công.</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
@@ -3205,7 +3217,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Các mutation aggregate Order–Payment–Inventory dùng transaction Serializable trên PostgreSQL. Lưu PROCESSING/REFUND_PENDING trước khi gọi gateway; finalize là transaction riêng. Gateway và DB không có distributed transaction, khoảng hở được reconciliation xử lý.</t>
+          <t>Mutation aggregate Order–Payment–Inventory chạy trong 1 transaction Serializable trên PostgreSQL; lưu PROCESSING/REFUND_PENDING trước khi gọi gateway, finalize là transaction thứ 2. Hệ thống dùng 0 distributed transaction; khoảng hở được 1 recovery worker đối soát.</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -3222,7 +3234,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Branch coverage tối thiểu 90% cho target đã đo: InputValidator và tập target fuzz được chọn. Coverage không đại diện toàn ứng dụng; ghi số đo và thời điểm từ coverage_summary.json/application_fuzzing.results.json.</t>
+          <t>Branch coverage tối thiểu 90% cho target đã đo. Snapshot 22/10/2026: InputValidator 97,22%, MoneyAmounts 100%, fuzz target 97,50% (3 target, không đại diện toàn ứng dụng).</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -3231,7 +3243,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28.8" customHeight="1">
+    <row r="4" ht="43.2" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>NFR-3</t>
@@ -3239,7 +3251,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Log lỗi phải đủ OrderId/UserId để truy vết nhưng không được ghi mật khẩu, JWT, Jwt:Key hoặc connection string.</t>
+          <t>Log lỗi chỉ dùng allowlist 8 trường (correlationId, orderId, userId, paymentId, event, status, errorCode, durationMs); 0 mật khẩu/JWT/Jwt:Key/connection string/raw body trong log và audit.</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -3256,7 +3268,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Secret và connection string phải được cung cấp ngoài source control; Jwt:Key phải có ít nhất 32 ký tự.</t>
+          <t>Secret và connection string nằm ngoài source control; Jwt:Key dài tối thiểu 32 ký tự (256-bit HS256), 0 secret hard-code trong repository.</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -3273,7 +3285,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Các bản C biên dịch với AddressSanitizer/UndefinedBehaviorSanitizer phải phát hiện đúng bản lỗi và không báo lỗi với bản FIXED trên cùng ca kiểm thử.</t>
+          <t>5 module C BUGGY/FIXED chạy 22/22 case sanitizer; bản BUGGY phải phát hiện đủ 5/5 lỗi (CWE-120/401/415/416), bản FIXED 0 báo cáo ASan/UBSan trên cùng input.</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -3282,7 +3294,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28.8" customHeight="1">
+    <row r="7" ht="43.2" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>NFR-6</t>
@@ -3290,7 +3302,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Pipeline kiểm chứng phải duyệt toàn bộ model hữu hạn, lưu counterexample cho model lỗi và ghi rõ bound, fairness, assumptions và giới hạn kết luận.</t>
+          <t>Pipeline kiểm chứng phải duyệt toàn bộ 14 state/35 event của model hữu hạn, kiểm 15 property và 6 mutation; lưu counterexample cho model lỗi, ghi rõ bound, fairness, assumptions và 0 kết luận vượt phạm vi.</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -3299,7 +3311,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="43.2" customHeight="1">
+    <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t>NFR-7</t>
@@ -3307,7 +3319,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Timeout wrapper charge/refund/status mặc định 5000ms, startup validate 50..60000ms. Caller không chờ vô hạn; late result không tự ghi state. Adapter không hợp tác chưa có cơ chế cưỡng chế dừng, backpressure vẫn là giới hạn.</t>
+          <t>Timeout wrapper charge/refund/status mặc định 5000ms; startup validate cấu hình trong khoảng 50..60000ms. 0 caller chờ vô hạn; late result không tự ghi state.</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -3316,7 +3328,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="43.2" customHeight="1">
+    <row r="9" ht="28.8" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>NFR-8</t>
@@ -3324,7 +3336,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>AuditEvents append-only chặn UPDATE/DELETE/TRUNCATE bằng PostgreSQL trigger; COMMIT audit chỉ bảo vệ Orders/Payments. Không chống DBA đổi schema/disable trigger; chưa có retention job hoặc chữ ký chống sửa log.</t>
+          <t>AuditEvents append-only bằng 4 PostgreSQL trigger chặn UPDATE/DELETE/TRUNCATE; 0 mutation audit được phép, COMMIT audit chỉ bảo vệ Orders/Payments.</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -3333,7 +3345,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="43.2" customHeight="1">
+    <row r="10" ht="28.8" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>NFR-9</t>
@@ -3341,7 +3353,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Kết quả nghiệm thu phải ghi total/pass/fail/skip, thời điểm, source/artifact hash khi có và giới hạn. Demo filtered tests không ghi đè summary toàn suite; snapshot evidence không là lần chạy mới.</t>
+          <t>Kết quả nghiệm thu ghi total/pass/fail/skip, thời điểm và hash artifact. Snapshot 22/10/2026: unit 149/149, integration 35/35, fail 0, skip 0.</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
@@ -3358,7 +3370,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Load/race phải kiểm no duplicate, conservation stock, bounded attempts và COMMIT count. Báo raw samples/p95/p99/status; workload hai API process hữu hạn và limiter local không chứng minh shared quota hoặc SLA production.</t>
+          <t>Load/race đo trên 2 API process, 8 user, 4 product và 96 logical request mỗi scenario; báo raw sample, p95, p99 và 0 duplicate charge/oversell trong workload đã chạy.</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
@@ -3505,7 +3517,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="43.2" customHeight="1">
+    <row r="8" ht="57.6" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t>CON-7</t>
@@ -3513,7 +3525,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Runtime MaxChargeAttempts=2. Model PAYMENT_PROCESSING_FINAL vẫn có cạnh final_payment_unknown/final_charged_but_commit_failed → PAYMENT_RETRY để giữ UNKNOWN; graph không mã hóa đầy đủ counter runtime và không là proof bound mọi đường thực thi.</t>
+          <t>Runtime MaxChargeAttempts=2. Model PAYMENT_PROCESSING_FINAL vẫn có cạnh stutter final_payment_unknown/final_charged_but_commit_failed → PAYMENT_RETRY để giữ UNKNOWN; workbook dùng progress projection (bỏ cạnh stutter) nên không tạo charge loop. Graph đầy đủ vẫn không chứng minh bound mọi đường thực thi.</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -3652,7 +3664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3696,7 +3708,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>created, inventory_unreserved, no_invalid_transition, no_resource_conflict</t>
+          <t>created, inventory_unreserved</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3718,7 +3730,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>validated, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>validated, inventory_reserved, amount_verified</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3740,12 +3752,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>payment_pending, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>payment_pending, inventory_reserved, amount_verified</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PAYMENT_PROCESSING, CANCELLED, PAYMENT_PENDING</t>
+          <t>PAYMENT_PROCESSING, CANCELLED</t>
         </is>
       </c>
     </row>
@@ -3762,12 +3774,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>payment_processing, inventory_reserved, amount_verified, payment_lock, no_invalid_transition, no_resource_conflict</t>
+          <t>payment_processing, inventory_reserved, amount_verified, payment_lock</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PAID, PAYMENT_RETRY, FAILED, PAYMENT_PROCESSING</t>
+          <t>PAID, PAYMENT_RETRY, FAILED</t>
         </is>
       </c>
     </row>
@@ -3784,12 +3796,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>payment_retry, inventory_reserved, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>payment_retry, inventory_reserved, amount_verified</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PAYMENT_PROCESSING_FINAL, PAYMENT_RETRY</t>
+          <t>PAYMENT_PROCESSING_FINAL</t>
         </is>
       </c>
     </row>
@@ -3806,12 +3818,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>payment_processing, final_retry, inventory_reserved, amount_verified, payment_lock, no_invalid_transition, no_resource_conflict</t>
+          <t>payment_processing, final_retry, inventory_reserved, amount_verified, payment_lock</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PAID, FAILED, PAYMENT_RETRY</t>
+          <t>PAID, FAILED</t>
         </is>
       </c>
     </row>
@@ -3828,19 +3840,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>paid, payment_success, amount_verified, inventory_reserved, no_invalid_transition, no_resource_conflict</t>
+          <t>paid, payment_success, amount_verified, inventory_reserved</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CONFIRMED, PAID, CONFIRMATION_RETRY, REFUND_PENDING</t>
+          <t>CONFIRMED, REFUND_PENDING</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CONFIRMATION_RETRY</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3850,19 +3862,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>paid, payment_success, confirmation_retry, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>confirmed, paid, payment_success, amount_verified</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CONFIRMED, REFUND_PENDING</t>
+          <t>COMPLETED, REFUND_PENDING</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CONFIRMED</t>
+          <t>REFUND_PENDING</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3872,19 +3884,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>confirmed, paid, payment_success, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>paid, payment_success, refund_pending, amount_verified</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COMPLETED, REFUND_PENDING</t>
+          <t>REFUNDED</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REFUND_PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3894,19 +3906,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>paid, payment_success, refund_pending, amount_verified, no_invalid_transition, no_resource_conflict</t>
+          <t>completed, paid, payment_success, amount_verified, terminal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>REFUNDED, REFUND_PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>COMPLETED</t>
+          <t>CANCELLED</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3916,19 +3928,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>completed, paid, payment_success, amount_verified, terminal, no_invalid_transition, no_resource_conflict</t>
+          <t>cancelled, inventory_released, terminal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMPLETED</t>
+          <t>CANCELLED</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CANCELLED</t>
+          <t>PRE_PAYMENT_REJECTED</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3938,19 +3950,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cancelled, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
+          <t>failed, pre_payment_failure, inventory_unreserved, terminal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CANCELLED</t>
+          <t>PRE_PAYMENT_REJECTED</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PRE_PAYMENT_REJECTED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3960,19 +3972,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>failed, pre_payment_failure, inventory_unreserved, terminal, no_invalid_transition, no_resource_conflict</t>
+          <t>failed, inventory_released, terminal</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PRE_PAYMENT_REJECTED</t>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>REFUNDED</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3982,34 +3994,100 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>failed, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
+          <t>refunded, payment_compensated, inventory_released, terminal</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>REFUNDED</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REFUNDED</t>
+          <t>free</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>main_holds, log_holds</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>main_holds</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>refunded, payment_compensated, inventory_released, terminal, no_invalid_transition, no_resource_conflict</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>REFUNDED</t>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>main_locked</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>free, conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>log_holds</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>log_locked</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>conflict</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>main_locked, log_locked, violation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>free</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="75" customWidth="1" min="1" max="1"/>
@@ -4040,47 +4118,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AG(no_invalid_transition)</t>
+          <t>AG(!violation)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AG(no_resource_conflict)</t>
+          <t>EF(main_locked)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EF(payment_processing)</t>
+          <t>AG(payment_pending -&gt; AF(paid | cancelled | failed))</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EF(payment_success)</t>
+          <t>AG(payment_processing -&gt; AF(paid | failed))</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EF(refund_pending)</t>
+          <t>AG(paid -&gt; AF(completed | refunded))</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EF(refunded)</t>
+          <t>AG(confirmed -&gt; AF(completed | refunded))</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>AG(refund_pending -&gt; AF(refunded))</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EF(payment_success)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EF(refunded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>EF(terminal)</t>
         </is>
@@ -4097,7 +4196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4119,12 +4218,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>main_locked</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>log_locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>payment_pending</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>payment_success</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>inventory_reserved</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>inventory_released</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4223,11 +4382,15 @@
           <t>buffer-overflow</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>31</v>
-      </c>
-      <c r="H2" t="n">
-        <v>32</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -4259,11 +4422,15 @@
           <t>buffer-overflow</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>31</v>
-      </c>
-      <c r="H3" t="n">
-        <v>32</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -4295,11 +4462,15 @@
           <t>use-after-free</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>101</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -4331,11 +4502,15 @@
           <t>memory-leak</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>5</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4367,11 +4542,91 @@
           <t>double-free</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>return_rate_ratio</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>divide</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>returned, borrowed</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>payment_override_code</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>magic_value</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>code_a, code_b</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>6284</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4917</v>
       </c>
     </row>
   </sheetData>
@@ -4419,117 +4674,117 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>order_item_subtotal_cents</t>
+          <t>order_total_cents</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>quantity, unit_price_cents</t>
+          <t>order_subtotal_cents, shipping_fee_cents</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1 &lt;= quantity &lt;= 10000 and 1 &lt;= unit_price_cents &lt;= 99999999 and quantity * unit_price_cents &gt; 2147483647</t>
+          <t>order_subtotal_cents &gt;= 0 and shipping_fee_cents &gt;= 0 and order_subtotal_cents + shipping_fee_cents &gt; 2000000000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>quantity * unit_price_cents</t>
+          <t>order_subtotal_cents + shipping_fee_cents</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>order_total_cents</t>
+          <t>payment_total_cents</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>subtotal1, subtotal2</t>
+          <t>payment1_cents, payment2_cents</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>subtotal1 &gt;= 0 and subtotal2 &gt;= 0 and subtotal1 + subtotal2 &gt; 2147483647</t>
+          <t>payment1_cents &gt;= 0 and payment2_cents &gt;= 0 and payment1_cents + payment2_cents &gt; 2000000000</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>subtotal1 + subtotal2</t>
+          <t>payment1_cents + payment2_cents</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>two_payment_total_cents</t>
+          <t>daily_order_counter</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>payment1_cents, payment2_cents</t>
+          <t>orders_today, orders_backlog</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>payment1_cents &gt;= 0 and payment2_cents &gt;= 0 and payment1_cents + payment2_cents &gt; 2147483647</t>
+          <t>orders_today &gt;= 0 and orders_backlog &gt;= 0 and orders_today + orders_backlog &gt; 32767</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>payment1_cents + payment2_cents</t>
+          <t>orders_today + orders_backlog</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>inventory_after_reserve</t>
+          <t>active_session_counter</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>stock, quantity</t>
+          <t>active_sessions, reserved_sessions</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0 &lt;= stock &lt;= 2147483647 and 1 &lt;= quantity &lt;= 10000 and stock - quantity &lt; 0</t>
+          <t>active_sessions &gt;= 0 and reserved_sessions &gt;= 0 and active_sessions + reserved_sessions &gt; 65535</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>stock - quantity</t>
+          <t>active_sessions + reserved_sessions</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>retry_counter_increment</t>
+          <t>backup_size_bytes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>retry_count, one</t>
+          <t>full_backup_bytes, incremental_bytes</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0 &lt;= retry_count &lt;= 2147483647 and one == 1 and retry_count + one &gt; 2147483647</t>
+          <t>full_backup_bytes &gt;= 0 and incremental_bytes &gt;= 0 and full_backup_bytes + incremental_bytes &gt; 4294967295</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>retry_count + one</t>
+          <t>full_backup_bytes + incremental_bytes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>refund_total_cents</t>
+          <t>refund_ledger_cents</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4539,7 +4794,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>paid_cents &gt;= 0 and refunded_cents &gt;= 0 and paid_cents + refunded_cents &gt; 2147483647</t>
+          <t>paid_cents &gt;= 0 and refunded_cents &gt;= 0 and paid_cents + refunded_cents &gt; 2000000000</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>